<commit_message>
Changed Esxcel spreadsheet again
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1843" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B403573-8B0C-475D-841F-A142B82FEBB3}"/>
+  <xr:revisionPtr revIDLastSave="1847" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4435021-B7F8-474A-9BF9-BB4AF9FD39CF}"/>
   <bookViews>
     <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1982,10 +1982,6 @@
 </FeaturePropertyBags>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -14530,7 +14526,7 @@
         <v>46196</v>
       </c>
       <c r="L91" s="20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M91" s="102" t="s">
         <v>333</v>

</xml_diff>

<commit_message>
Added overdue and upcoming to the reticulation
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1847" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4435021-B7F8-474A-9BF9-BB4AF9FD39CF}"/>
+  <xr:revisionPtr revIDLastSave="1848" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3777CD5-27F2-44C3-B7E1-1FC4C2C0108B}"/>
   <bookViews>
-    <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Water meters " sheetId="1" r:id="rId1"/>
@@ -9971,7 +9971,7 @@
         <v>46171</v>
       </c>
       <c r="I192" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J192" s="101" t="s">
         <v>332</v>

</xml_diff>

<commit_message>
NEw wtaer meters installed
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1848" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3777CD5-27F2-44C3-B7E1-1FC4C2C0108B}"/>
+  <xr:revisionPtr revIDLastSave="1854" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4E23647-6F74-49CD-AA94-8763423563C4}"/>
   <bookViews>
     <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3032" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3034" uniqueCount="371">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -1152,6 +1152,12 @@
   </si>
   <si>
     <t>MS2</t>
+  </si>
+  <si>
+    <t>10192050</t>
+  </si>
+  <si>
+    <t>10216099</t>
   </si>
 </sst>
 </file>
@@ -4072,7 +4078,9 @@
       <c r="B48" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="C48" s="83"/>
+      <c r="C48" s="83" t="s">
+        <v>370</v>
+      </c>
       <c r="D48" s="83" t="s">
         <v>11</v>
       </c>
@@ -4082,8 +4090,12 @@
       <c r="F48" s="83" t="s">
         <v>13</v>
       </c>
-      <c r="G48" s="6"/>
-      <c r="H48" s="6"/>
+      <c r="G48" s="6">
+        <v>0.154</v>
+      </c>
+      <c r="H48" s="88">
+        <v>46204</v>
+      </c>
       <c r="I48" s="32" t="b">
         <v>0</v>
       </c>
@@ -4148,7 +4160,9 @@
       <c r="B50" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="C50" s="83"/>
+      <c r="C50" s="83" t="s">
+        <v>369</v>
+      </c>
       <c r="D50" s="83" t="s">
         <v>11</v>
       </c>
@@ -4158,8 +4172,12 @@
       <c r="F50" s="83" t="s">
         <v>13</v>
       </c>
-      <c r="G50" s="6"/>
-      <c r="H50" s="6"/>
+      <c r="G50" s="6">
+        <v>6.8000000000000005E-2</v>
+      </c>
+      <c r="H50" s="88">
+        <v>46204</v>
+      </c>
       <c r="I50" s="32" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Water meter AMR loaded update excel
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1854" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4E23647-6F74-49CD-AA94-8763423563C4}"/>
+  <xr:revisionPtr revIDLastSave="1868" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E1B29A8-BC26-43B7-A66B-F0BC8E2358CE}"/>
   <bookViews>
     <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4097,7 +4097,7 @@
         <v>46204</v>
       </c>
       <c r="I48" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J48" s="101" t="s">
         <v>344</v>
@@ -4179,7 +4179,7 @@
         <v>46204</v>
       </c>
       <c r="I50" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J50" s="101" t="s">
         <v>344</v>
@@ -4261,7 +4261,7 @@
         <v>46204</v>
       </c>
       <c r="I52" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J52" s="101" t="s">
         <v>344</v>
@@ -4343,7 +4343,7 @@
         <v>46204</v>
       </c>
       <c r="I54" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J54" s="101" t="s">
         <v>344</v>
@@ -4425,7 +4425,7 @@
         <v>46204</v>
       </c>
       <c r="I56" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J56" s="101" t="s">
         <v>344</v>
@@ -4507,7 +4507,7 @@
         <v>46204</v>
       </c>
       <c r="I58" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J58" s="101" t="s">
         <v>344</v>
@@ -4589,7 +4589,7 @@
         <v>46204</v>
       </c>
       <c r="I60" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J60" s="101" t="s">
         <v>344</v>
@@ -4891,7 +4891,7 @@
         <v>46204</v>
       </c>
       <c r="I67" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J67" s="101" t="s">
         <v>346</v>
@@ -4979,7 +4979,7 @@
         <v>46204</v>
       </c>
       <c r="I69" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J69" s="101" t="s">
         <v>346</v>
@@ -5815,7 +5815,7 @@
         <v>46204</v>
       </c>
       <c r="I88" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J88" s="101" t="s">
         <v>333</v>

</xml_diff>

<commit_message>
New water meter installed
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1868" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E1B29A8-BC26-43B7-A66B-F0BC8E2358CE}"/>
+  <xr:revisionPtr revIDLastSave="1875" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2A4FA20-61AD-4BA3-AAC3-F04073678DBF}"/>
   <bookViews>
     <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3034" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3035" uniqueCount="373">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -1158,6 +1158,12 @@
   </si>
   <si>
     <t>10216099</t>
+  </si>
+  <si>
+    <t>20mm</t>
+  </si>
+  <si>
+    <t>9993270</t>
   </si>
 </sst>
 </file>
@@ -2338,7 +2344,7 @@
         <v>12</v>
       </c>
       <c r="F2" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -2376,7 +2382,7 @@
         <v>12</v>
       </c>
       <c r="F3" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -2414,7 +2420,7 @@
         <v>12</v>
       </c>
       <c r="F4" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
@@ -2452,7 +2458,7 @@
         <v>12</v>
       </c>
       <c r="F5" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -2490,7 +2496,7 @@
         <v>12</v>
       </c>
       <c r="F6" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -2528,7 +2534,7 @@
         <v>12</v>
       </c>
       <c r="F7" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
@@ -2566,7 +2572,7 @@
         <v>12</v>
       </c>
       <c r="F8" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
@@ -2604,7 +2610,7 @@
         <v>12</v>
       </c>
       <c r="F9" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
@@ -2642,7 +2648,7 @@
         <v>12</v>
       </c>
       <c r="F10" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
@@ -2680,7 +2686,7 @@
         <v>12</v>
       </c>
       <c r="F11" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
@@ -2718,7 +2724,7 @@
         <v>12</v>
       </c>
       <c r="F12" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
@@ -2756,7 +2762,7 @@
         <v>12</v>
       </c>
       <c r="F13" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
@@ -2794,7 +2800,7 @@
         <v>12</v>
       </c>
       <c r="F14" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
@@ -2832,7 +2838,7 @@
         <v>12</v>
       </c>
       <c r="F15" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
@@ -2870,7 +2876,7 @@
         <v>12</v>
       </c>
       <c r="F16" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
@@ -2908,7 +2914,7 @@
         <v>12</v>
       </c>
       <c r="F17" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
@@ -2946,7 +2952,7 @@
         <v>12</v>
       </c>
       <c r="F18" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
@@ -2984,7 +2990,7 @@
         <v>12</v>
       </c>
       <c r="F19" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
@@ -3022,7 +3028,7 @@
         <v>12</v>
       </c>
       <c r="F20" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
@@ -3060,7 +3066,7 @@
         <v>12</v>
       </c>
       <c r="F21" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
@@ -3098,7 +3104,7 @@
         <v>12</v>
       </c>
       <c r="F22" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
@@ -3136,7 +3142,7 @@
         <v>12</v>
       </c>
       <c r="F23" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
@@ -3174,7 +3180,7 @@
         <v>12</v>
       </c>
       <c r="F24" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
@@ -3212,7 +3218,7 @@
         <v>12</v>
       </c>
       <c r="F25" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
@@ -3250,7 +3256,7 @@
         <v>12</v>
       </c>
       <c r="F26" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
@@ -3288,7 +3294,7 @@
         <v>12</v>
       </c>
       <c r="F27" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
@@ -3326,7 +3332,7 @@
         <v>12</v>
       </c>
       <c r="F28" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
@@ -3364,7 +3370,7 @@
         <v>12</v>
       </c>
       <c r="F29" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
@@ -3402,7 +3408,7 @@
         <v>12</v>
       </c>
       <c r="F30" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
@@ -3440,7 +3446,7 @@
         <v>12</v>
       </c>
       <c r="F31" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
@@ -3478,7 +3484,7 @@
         <v>12</v>
       </c>
       <c r="F32" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G32" s="6"/>
       <c r="H32" s="6"/>
@@ -3516,7 +3522,7 @@
         <v>12</v>
       </c>
       <c r="F33" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G33" s="6"/>
       <c r="H33" s="6"/>
@@ -3554,7 +3560,7 @@
         <v>12</v>
       </c>
       <c r="F34" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G34" s="6"/>
       <c r="H34" s="6"/>
@@ -3592,7 +3598,7 @@
         <v>12</v>
       </c>
       <c r="F35" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
@@ -3630,7 +3636,7 @@
         <v>12</v>
       </c>
       <c r="F36" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
@@ -3668,7 +3674,7 @@
         <v>12</v>
       </c>
       <c r="F37" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="6"/>
@@ -3706,7 +3712,7 @@
         <v>12</v>
       </c>
       <c r="F38" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G38" s="6"/>
       <c r="H38" s="6"/>
@@ -3744,7 +3750,7 @@
         <v>12</v>
       </c>
       <c r="F39" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G39" s="6"/>
       <c r="H39" s="6"/>
@@ -3782,7 +3788,7 @@
         <v>12</v>
       </c>
       <c r="F40" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G40" s="6"/>
       <c r="H40" s="6"/>
@@ -3820,7 +3826,7 @@
         <v>12</v>
       </c>
       <c r="F41" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
@@ -3858,7 +3864,7 @@
         <v>12</v>
       </c>
       <c r="F42" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
@@ -3896,7 +3902,7 @@
         <v>12</v>
       </c>
       <c r="F43" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
@@ -3934,7 +3940,7 @@
         <v>12</v>
       </c>
       <c r="F44" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
@@ -3972,7 +3978,7 @@
         <v>12</v>
       </c>
       <c r="F45" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G45" s="6"/>
       <c r="H45" s="6"/>
@@ -4010,7 +4016,7 @@
         <v>12</v>
       </c>
       <c r="F46" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G46" s="6"/>
       <c r="H46" s="6"/>
@@ -4048,7 +4054,7 @@
         <v>12</v>
       </c>
       <c r="F47" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G47" s="6"/>
       <c r="H47" s="6"/>
@@ -4088,7 +4094,7 @@
         <v>12</v>
       </c>
       <c r="F48" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G48" s="6">
         <v>0.154</v>
@@ -4130,7 +4136,7 @@
         <v>12</v>
       </c>
       <c r="F49" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G49" s="6"/>
       <c r="H49" s="6"/>
@@ -4170,7 +4176,7 @@
         <v>12</v>
       </c>
       <c r="F50" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G50" s="6">
         <v>6.8000000000000005E-2</v>
@@ -4212,7 +4218,7 @@
         <v>12</v>
       </c>
       <c r="F51" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G51" s="6"/>
       <c r="H51" s="6"/>
@@ -4252,7 +4258,7 @@
         <v>12</v>
       </c>
       <c r="F52" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G52" s="6">
         <v>8.8999999999999996E-2</v>
@@ -4294,7 +4300,7 @@
         <v>12</v>
       </c>
       <c r="F53" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G53" s="6"/>
       <c r="H53" s="6"/>
@@ -4334,7 +4340,7 @@
         <v>12</v>
       </c>
       <c r="F54" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G54" s="6">
         <v>6.7000000000000004E-2</v>
@@ -4376,7 +4382,7 @@
         <v>12</v>
       </c>
       <c r="F55" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G55" s="6"/>
       <c r="H55" s="6"/>
@@ -4416,7 +4422,7 @@
         <v>12</v>
       </c>
       <c r="F56" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G56" s="6">
         <v>9.0999999999999998E-2</v>
@@ -4458,7 +4464,7 @@
         <v>12</v>
       </c>
       <c r="F57" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G57" s="6"/>
       <c r="H57" s="6"/>
@@ -4498,7 +4504,7 @@
         <v>12</v>
       </c>
       <c r="F58" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G58" s="6">
         <v>7.5999999999999998E-2</v>
@@ -4540,7 +4546,7 @@
         <v>12</v>
       </c>
       <c r="F59" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G59" s="6"/>
       <c r="H59" s="6"/>
@@ -4580,7 +4586,7 @@
         <v>12</v>
       </c>
       <c r="F60" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G60" s="6">
         <v>8.2000000000000003E-2</v>
@@ -4614,7 +4620,9 @@
       <c r="B61" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="C61" s="83"/>
+      <c r="C61" s="83" t="s">
+        <v>372</v>
+      </c>
       <c r="D61" s="83" t="s">
         <v>11</v>
       </c>
@@ -4622,12 +4630,16 @@
         <v>12</v>
       </c>
       <c r="F61" s="83" t="s">
-        <v>13</v>
-      </c>
-      <c r="G61" s="6"/>
-      <c r="H61" s="6"/>
+        <v>371</v>
+      </c>
+      <c r="G61" s="6">
+        <v>8.1000000000000003E-2</v>
+      </c>
+      <c r="H61" s="88">
+        <v>46205</v>
+      </c>
       <c r="I61" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J61" s="101" t="s">
         <v>347</v>
@@ -4662,7 +4674,7 @@
         <v>12</v>
       </c>
       <c r="F62" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G62" s="6">
         <v>6.7000000000000004E-2</v>
@@ -4706,7 +4718,7 @@
         <v>12</v>
       </c>
       <c r="F63" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G63" s="6">
         <v>7.3999999999999996E-2</v>
@@ -4750,7 +4762,7 @@
         <v>12</v>
       </c>
       <c r="F64" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G64" s="6">
         <v>6.6000000000000003E-2</v>
@@ -4794,7 +4806,7 @@
         <v>12</v>
       </c>
       <c r="F65" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G65" s="6">
         <v>8.1000000000000003E-2</v>
@@ -4838,7 +4850,7 @@
         <v>12</v>
       </c>
       <c r="F66" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G66" s="6">
         <v>6.7000000000000004E-2</v>
@@ -4882,7 +4894,7 @@
         <v>12</v>
       </c>
       <c r="F67" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G67" s="6">
         <v>8.2000000000000003E-2</v>
@@ -4926,7 +4938,7 @@
         <v>12</v>
       </c>
       <c r="F68" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G68" s="6">
         <v>6.5000000000000002E-2</v>
@@ -4970,7 +4982,7 @@
         <v>12</v>
       </c>
       <c r="F69" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G69" s="6">
         <v>6.9000000000000006E-2</v>
@@ -5014,7 +5026,7 @@
         <v>12</v>
       </c>
       <c r="F70" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G70" s="6">
         <v>6.6000000000000003E-2</v>
@@ -5058,7 +5070,7 @@
         <v>12</v>
       </c>
       <c r="F71" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G71" s="6">
         <v>7.1999999999999995E-2</v>
@@ -5102,7 +5114,7 @@
         <v>12</v>
       </c>
       <c r="F72" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G72" s="6">
         <v>8.3000000000000004E-2</v>
@@ -5146,7 +5158,7 @@
         <v>12</v>
       </c>
       <c r="F73" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G73" s="6">
         <v>4.2000000000000003E-2</v>
@@ -5190,7 +5202,7 @@
         <v>12</v>
       </c>
       <c r="F74" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G74" s="6">
         <v>7.0000000000000007E-2</v>
@@ -5234,7 +5246,7 @@
         <v>12</v>
       </c>
       <c r="F75" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G75" s="6">
         <v>7.0000000000000007E-2</v>
@@ -5278,7 +5290,7 @@
         <v>12</v>
       </c>
       <c r="F76" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G76" s="6">
         <v>7.1999999999999995E-2</v>
@@ -5322,7 +5334,7 @@
         <v>12</v>
       </c>
       <c r="F77" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G77" s="6">
         <v>0.10199999999999999</v>
@@ -5366,7 +5378,7 @@
         <v>12</v>
       </c>
       <c r="F78" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G78" s="6">
         <v>0.10299999999999999</v>
@@ -5410,7 +5422,7 @@
         <v>12</v>
       </c>
       <c r="F79" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G79" s="6">
         <v>0.10299999999999999</v>
@@ -5454,7 +5466,7 @@
         <v>12</v>
       </c>
       <c r="F80" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G80" s="6">
         <v>9.7000000000000003E-2</v>
@@ -5498,7 +5510,7 @@
         <v>12</v>
       </c>
       <c r="F81" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G81" s="6">
         <v>9.6000000000000002E-2</v>
@@ -5542,7 +5554,7 @@
         <v>12</v>
       </c>
       <c r="F82" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G82" s="6">
         <v>0.10199999999999999</v>
@@ -5586,7 +5598,7 @@
         <v>12</v>
       </c>
       <c r="F83" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G83" s="6">
         <v>0.10199999999999999</v>
@@ -5630,7 +5642,7 @@
         <v>12</v>
       </c>
       <c r="F84" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G84" s="6">
         <v>0.10199999999999999</v>
@@ -5674,7 +5686,7 @@
         <v>12</v>
       </c>
       <c r="F85" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G85" s="6">
         <v>0.10199999999999999</v>
@@ -5718,7 +5730,7 @@
         <v>12</v>
       </c>
       <c r="F86" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G86" s="6">
         <v>0.10100000000000001</v>
@@ -5762,7 +5774,7 @@
         <v>12</v>
       </c>
       <c r="F87" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G87" s="6">
         <v>8.7999999999999995E-2</v>
@@ -5806,7 +5818,7 @@
         <v>12</v>
       </c>
       <c r="F88" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G88" s="6">
         <v>6.9000000000000006E-2</v>
@@ -5850,7 +5862,7 @@
         <v>12</v>
       </c>
       <c r="F89" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G89" s="6">
         <v>8.5000000000000006E-2</v>
@@ -5894,7 +5906,7 @@
         <v>12</v>
       </c>
       <c r="F90" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G90" s="6">
         <v>0.10199999999999999</v>
@@ -5938,7 +5950,7 @@
         <v>12</v>
       </c>
       <c r="F91" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G91" s="6">
         <v>9.7000000000000003E-2</v>
@@ -5982,7 +5994,7 @@
         <v>12</v>
       </c>
       <c r="F92" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G92" s="6">
         <v>9.9000000000000005E-2</v>
@@ -6026,7 +6038,7 @@
         <v>12</v>
       </c>
       <c r="F93" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G93" s="6">
         <v>0.10199999999999999</v>
@@ -6070,7 +6082,7 @@
         <v>12</v>
       </c>
       <c r="F94" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G94" s="6">
         <v>9.5000000000000001E-2</v>
@@ -6114,7 +6126,7 @@
         <v>12</v>
       </c>
       <c r="F95" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G95" s="6">
         <v>8.5999999999999993E-2</v>
@@ -6158,7 +6170,7 @@
         <v>12</v>
       </c>
       <c r="F96" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G96" s="6">
         <v>0.104</v>
@@ -6202,7 +6214,7 @@
         <v>12</v>
       </c>
       <c r="F97" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G97" s="6">
         <v>8.5999999999999993E-2</v>
@@ -6246,7 +6258,7 @@
         <v>12</v>
       </c>
       <c r="F98" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G98" s="6">
         <v>9.9000000000000005E-2</v>
@@ -6290,7 +6302,7 @@
         <v>12</v>
       </c>
       <c r="F99" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G99" s="6">
         <v>0.10199999999999999</v>
@@ -6334,7 +6346,7 @@
         <v>12</v>
       </c>
       <c r="F100" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G100" s="6">
         <v>0.10100000000000001</v>
@@ -6378,7 +6390,7 @@
         <v>12</v>
       </c>
       <c r="F101" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G101" s="6">
         <v>0.10199999999999999</v>
@@ -6422,7 +6434,7 @@
         <v>12</v>
       </c>
       <c r="F102" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G102" s="6">
         <v>9.0999999999999998E-2</v>
@@ -6466,7 +6478,7 @@
         <v>12</v>
       </c>
       <c r="F103" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G103" s="6">
         <v>0.105</v>
@@ -6510,7 +6522,7 @@
         <v>12</v>
       </c>
       <c r="F104" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G104" s="6">
         <v>7.2999999999999995E-2</v>
@@ -6552,7 +6564,7 @@
         <v>12</v>
       </c>
       <c r="F105" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G105" s="6"/>
       <c r="H105" s="6"/>
@@ -6592,7 +6604,7 @@
         <v>12</v>
       </c>
       <c r="F106" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G106" s="6">
         <v>9.2999999999999999E-2</v>
@@ -6634,7 +6646,7 @@
         <v>12</v>
       </c>
       <c r="F107" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G107" s="6"/>
       <c r="H107" s="6"/>
@@ -6674,7 +6686,7 @@
         <v>12</v>
       </c>
       <c r="F108" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G108" s="6">
         <v>8.1000000000000003E-2</v>
@@ -6716,7 +6728,7 @@
         <v>12</v>
       </c>
       <c r="F109" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G109" s="6"/>
       <c r="H109" s="6"/>
@@ -6756,7 +6768,7 @@
         <v>12</v>
       </c>
       <c r="F110" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G110" s="6">
         <v>7.0999999999999994E-2</v>
@@ -6798,7 +6810,7 @@
         <v>12</v>
       </c>
       <c r="F111" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G111" s="6"/>
       <c r="H111" s="6"/>
@@ -6838,7 +6850,7 @@
         <v>12</v>
       </c>
       <c r="F112" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G112" s="6">
         <v>6.8000000000000005E-2</v>
@@ -6880,7 +6892,7 @@
         <v>12</v>
       </c>
       <c r="F113" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G113" s="6"/>
       <c r="H113" s="6"/>
@@ -6920,7 +6932,7 @@
         <v>12</v>
       </c>
       <c r="F114" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G114" s="6">
         <v>9.0999999999999998E-2</v>
@@ -6962,7 +6974,7 @@
         <v>12</v>
       </c>
       <c r="F115" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G115" s="6"/>
       <c r="H115" s="6"/>
@@ -7002,7 +7014,7 @@
         <v>12</v>
       </c>
       <c r="F116" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G116" s="6">
         <v>9.2999999999999999E-2</v>
@@ -7044,7 +7056,7 @@
         <v>12</v>
       </c>
       <c r="F117" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G117" s="6"/>
       <c r="H117" s="6"/>
@@ -7084,7 +7096,7 @@
         <v>12</v>
       </c>
       <c r="F118" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G118" s="6">
         <v>8.2000000000000003E-2</v>
@@ -7126,7 +7138,7 @@
         <v>12</v>
       </c>
       <c r="F119" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G119" s="6"/>
       <c r="H119" s="6"/>
@@ -7166,7 +7178,7 @@
         <v>12</v>
       </c>
       <c r="F120" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G120" s="6">
         <v>0.223</v>
@@ -7208,7 +7220,7 @@
         <v>12</v>
       </c>
       <c r="F121" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G121" s="6"/>
       <c r="H121" s="6"/>
@@ -7248,7 +7260,7 @@
         <v>12</v>
       </c>
       <c r="F122" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G122" s="6">
         <v>0.08</v>
@@ -7290,7 +7302,7 @@
         <v>12</v>
       </c>
       <c r="F123" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G123" s="6"/>
       <c r="H123" s="6"/>
@@ -7330,7 +7342,7 @@
         <v>12</v>
       </c>
       <c r="F124" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G124" s="6">
         <v>7.0999999999999994E-2</v>
@@ -7372,7 +7384,7 @@
         <v>12</v>
       </c>
       <c r="F125" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G125" s="6"/>
       <c r="H125" s="6"/>
@@ -7412,7 +7424,7 @@
         <v>12</v>
       </c>
       <c r="F126" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G126" s="6">
         <v>1.163</v>
@@ -7454,7 +7466,7 @@
         <v>12</v>
       </c>
       <c r="F127" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G127" s="6"/>
       <c r="H127" s="6"/>
@@ -7494,7 +7506,7 @@
         <v>12</v>
       </c>
       <c r="F128" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G128" s="6">
         <v>7.5999999999999998E-2</v>
@@ -7536,7 +7548,7 @@
         <v>12</v>
       </c>
       <c r="F129" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G129" s="6"/>
       <c r="H129" s="6"/>
@@ -7574,7 +7586,7 @@
         <v>12</v>
       </c>
       <c r="F130" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G130" s="6"/>
       <c r="H130" s="6"/>
@@ -7612,7 +7624,7 @@
         <v>12</v>
       </c>
       <c r="F131" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G131" s="6"/>
       <c r="H131" s="6"/>
@@ -7650,7 +7662,7 @@
         <v>12</v>
       </c>
       <c r="F132" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G132" s="6"/>
       <c r="H132" s="6"/>
@@ -7688,7 +7700,7 @@
         <v>12</v>
       </c>
       <c r="F133" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G133" s="6"/>
       <c r="H133" s="6"/>
@@ -7726,7 +7738,7 @@
         <v>12</v>
       </c>
       <c r="F134" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G134" s="6"/>
       <c r="H134" s="6"/>
@@ -7764,7 +7776,7 @@
         <v>12</v>
       </c>
       <c r="F135" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G135" s="6"/>
       <c r="H135" s="6"/>
@@ -7802,7 +7814,7 @@
         <v>12</v>
       </c>
       <c r="F136" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G136" s="6"/>
       <c r="H136" s="6"/>
@@ -7840,7 +7852,7 @@
         <v>12</v>
       </c>
       <c r="F137" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G137" s="6"/>
       <c r="H137" s="6"/>
@@ -7878,7 +7890,7 @@
         <v>12</v>
       </c>
       <c r="F138" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G138" s="6"/>
       <c r="H138" s="6"/>
@@ -7916,7 +7928,7 @@
         <v>12</v>
       </c>
       <c r="F139" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G139" s="6"/>
       <c r="H139" s="6"/>
@@ -7954,7 +7966,7 @@
         <v>12</v>
       </c>
       <c r="F140" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G140" s="6"/>
       <c r="H140" s="6"/>
@@ -7992,7 +8004,7 @@
         <v>12</v>
       </c>
       <c r="F141" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G141" s="6"/>
       <c r="H141" s="6"/>
@@ -8030,7 +8042,7 @@
         <v>12</v>
       </c>
       <c r="F142" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G142" s="6"/>
       <c r="H142" s="6"/>
@@ -8068,7 +8080,7 @@
         <v>12</v>
       </c>
       <c r="F143" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G143" s="6"/>
       <c r="H143" s="6"/>
@@ -8106,7 +8118,7 @@
         <v>12</v>
       </c>
       <c r="F144" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G144" s="6"/>
       <c r="H144" s="6"/>
@@ -8144,7 +8156,7 @@
         <v>12</v>
       </c>
       <c r="F145" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G145" s="6"/>
       <c r="H145" s="6"/>
@@ -8182,7 +8194,7 @@
         <v>12</v>
       </c>
       <c r="F146" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G146" s="6"/>
       <c r="H146" s="6"/>
@@ -8220,7 +8232,7 @@
         <v>12</v>
       </c>
       <c r="F147" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G147" s="6"/>
       <c r="H147" s="6"/>
@@ -8258,7 +8270,7 @@
         <v>12</v>
       </c>
       <c r="F148" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G148" s="6"/>
       <c r="H148" s="6"/>
@@ -8296,7 +8308,7 @@
         <v>12</v>
       </c>
       <c r="F149" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G149" s="6"/>
       <c r="H149" s="6"/>
@@ -8334,7 +8346,7 @@
         <v>12</v>
       </c>
       <c r="F150" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G150" s="6"/>
       <c r="H150" s="6"/>
@@ -8372,7 +8384,7 @@
         <v>12</v>
       </c>
       <c r="F151" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G151" s="6"/>
       <c r="H151" s="6"/>
@@ -8410,7 +8422,7 @@
         <v>12</v>
       </c>
       <c r="F152" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G152" s="6"/>
       <c r="H152" s="6"/>
@@ -8448,7 +8460,7 @@
         <v>12</v>
       </c>
       <c r="F153" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G153" s="6"/>
       <c r="H153" s="6"/>
@@ -8486,7 +8498,7 @@
         <v>12</v>
       </c>
       <c r="F154" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G154" s="6"/>
       <c r="H154" s="6"/>
@@ -8524,7 +8536,7 @@
         <v>12</v>
       </c>
       <c r="F155" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G155" s="6"/>
       <c r="H155" s="6"/>
@@ -8562,7 +8574,7 @@
         <v>12</v>
       </c>
       <c r="F156" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G156" s="6"/>
       <c r="H156" s="6"/>
@@ -8600,7 +8612,7 @@
         <v>12</v>
       </c>
       <c r="F157" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G157" s="6"/>
       <c r="H157" s="6"/>
@@ -8638,7 +8650,7 @@
         <v>12</v>
       </c>
       <c r="F158" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G158" s="6"/>
       <c r="H158" s="6"/>
@@ -8676,7 +8688,7 @@
         <v>12</v>
       </c>
       <c r="F159" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G159" s="6"/>
       <c r="H159" s="6"/>
@@ -8714,7 +8726,7 @@
         <v>12</v>
       </c>
       <c r="F160" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G160" s="6"/>
       <c r="H160" s="6"/>
@@ -8752,7 +8764,7 @@
         <v>12</v>
       </c>
       <c r="F161" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G161" s="6"/>
       <c r="H161" s="6"/>
@@ -8790,7 +8802,7 @@
         <v>12</v>
       </c>
       <c r="F162" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G162" s="6"/>
       <c r="H162" s="6"/>
@@ -8828,7 +8840,7 @@
         <v>12</v>
       </c>
       <c r="F163" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G163" s="6"/>
       <c r="H163" s="6"/>
@@ -8866,7 +8878,7 @@
         <v>12</v>
       </c>
       <c r="F164" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G164" s="6"/>
       <c r="H164" s="6"/>
@@ -8904,7 +8916,7 @@
         <v>12</v>
       </c>
       <c r="F165" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G165" s="6"/>
       <c r="H165" s="6"/>
@@ -8942,7 +8954,7 @@
         <v>12</v>
       </c>
       <c r="F166" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G166" s="6"/>
       <c r="H166" s="6"/>
@@ -8980,7 +8992,7 @@
         <v>12</v>
       </c>
       <c r="F167" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G167" s="6"/>
       <c r="H167" s="6"/>
@@ -9018,7 +9030,7 @@
         <v>12</v>
       </c>
       <c r="F168" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G168" s="6"/>
       <c r="H168" s="6"/>
@@ -9056,7 +9068,7 @@
         <v>12</v>
       </c>
       <c r="F169" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G169" s="6"/>
       <c r="H169" s="6"/>
@@ -9094,7 +9106,7 @@
         <v>12</v>
       </c>
       <c r="F170" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G170" s="6"/>
       <c r="H170" s="6"/>
@@ -9132,7 +9144,7 @@
         <v>12</v>
       </c>
       <c r="F171" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G171" s="6"/>
       <c r="H171" s="6"/>
@@ -9170,7 +9182,7 @@
         <v>12</v>
       </c>
       <c r="F172" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G172" s="6"/>
       <c r="H172" s="6"/>
@@ -9208,7 +9220,7 @@
         <v>12</v>
       </c>
       <c r="F173" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G173" s="6"/>
       <c r="H173" s="6"/>
@@ -9246,7 +9258,7 @@
         <v>12</v>
       </c>
       <c r="F174" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G174" s="6"/>
       <c r="H174" s="6"/>
@@ -9284,7 +9296,7 @@
         <v>12</v>
       </c>
       <c r="F175" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G175" s="6"/>
       <c r="H175" s="6"/>
@@ -9322,7 +9334,7 @@
         <v>12</v>
       </c>
       <c r="F176" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G176" s="6"/>
       <c r="H176" s="6"/>
@@ -9360,7 +9372,7 @@
         <v>12</v>
       </c>
       <c r="F177" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G177" s="6"/>
       <c r="H177" s="6"/>
@@ -9398,7 +9410,7 @@
         <v>12</v>
       </c>
       <c r="F178" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G178" s="6"/>
       <c r="H178" s="6"/>
@@ -9436,7 +9448,7 @@
         <v>12</v>
       </c>
       <c r="F179" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G179" s="6"/>
       <c r="H179" s="6"/>
@@ -9474,7 +9486,7 @@
         <v>12</v>
       </c>
       <c r="F180" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G180" s="6"/>
       <c r="H180" s="6"/>
@@ -9512,7 +9524,7 @@
         <v>12</v>
       </c>
       <c r="F181" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G181" s="6"/>
       <c r="H181" s="6"/>
@@ -9550,7 +9562,7 @@
         <v>12</v>
       </c>
       <c r="F182" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G182" s="6"/>
       <c r="H182" s="6"/>
@@ -9588,7 +9600,7 @@
         <v>12</v>
       </c>
       <c r="F183" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G183" s="6"/>
       <c r="H183" s="6"/>
@@ -9628,7 +9640,7 @@
         <v>12</v>
       </c>
       <c r="F184" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G184" s="6">
         <v>7.4999999999999997E-2</v>
@@ -9672,7 +9684,7 @@
         <v>12</v>
       </c>
       <c r="F185" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G185" s="6">
         <v>6.7000000000000004E-2</v>
@@ -9716,7 +9728,7 @@
         <v>12</v>
       </c>
       <c r="F186" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G186" s="6">
         <v>6.7000000000000004E-2</v>
@@ -9760,7 +9772,7 @@
         <v>12</v>
       </c>
       <c r="F187" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G187" s="6">
         <v>6.6000000000000003E-2</v>
@@ -9804,7 +9816,7 @@
         <v>12</v>
       </c>
       <c r="F188" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G188" s="6">
         <v>6.9000000000000006E-2</v>
@@ -9848,7 +9860,7 @@
         <v>12</v>
       </c>
       <c r="F189" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G189" s="6">
         <v>6.8000000000000005E-2</v>
@@ -9892,7 +9904,7 @@
         <v>12</v>
       </c>
       <c r="F190" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G190" s="6">
         <v>8.6999999999999994E-2</v>
@@ -9936,7 +9948,7 @@
         <v>12</v>
       </c>
       <c r="F191" s="83" t="s">
-        <v>13</v>
+        <v>371</v>
       </c>
       <c r="G191" s="6">
         <v>6.9000000000000006E-2</v>

</xml_diff>

<commit_message>
New water meters installed
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1875" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2A4FA20-61AD-4BA3-AAC3-F04073678DBF}"/>
+  <xr:revisionPtr revIDLastSave="1891" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D8C9523-006E-440A-ACCC-19308917722B}"/>
   <bookViews>
     <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3035" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3039" uniqueCount="377">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -1164,6 +1164,18 @@
   </si>
   <si>
     <t>9993270</t>
+  </si>
+  <si>
+    <t>9993264</t>
+  </si>
+  <si>
+    <t>10192024</t>
+  </si>
+  <si>
+    <t>9993269</t>
+  </si>
+  <si>
+    <t>9993263</t>
   </si>
 </sst>
 </file>
@@ -4292,7 +4304,9 @@
       <c r="B53" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="C53" s="83"/>
+      <c r="C53" s="83" t="s">
+        <v>376</v>
+      </c>
       <c r="D53" s="83" t="s">
         <v>11</v>
       </c>
@@ -4302,10 +4316,14 @@
       <c r="F53" s="83" t="s">
         <v>371</v>
       </c>
-      <c r="G53" s="6"/>
-      <c r="H53" s="6"/>
+      <c r="G53" s="6">
+        <v>7.5999999999999998E-2</v>
+      </c>
+      <c r="H53" s="88">
+        <v>46205</v>
+      </c>
       <c r="I53" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J53" s="101" t="s">
         <v>347</v>
@@ -4374,7 +4392,9 @@
       <c r="B55" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="C55" s="83"/>
+      <c r="C55" s="83" t="s">
+        <v>375</v>
+      </c>
       <c r="D55" s="83" t="s">
         <v>11</v>
       </c>
@@ -4384,10 +4404,14 @@
       <c r="F55" s="83" t="s">
         <v>371</v>
       </c>
-      <c r="G55" s="6"/>
-      <c r="H55" s="6"/>
+      <c r="G55" s="6">
+        <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="H55" s="88">
+        <v>46205</v>
+      </c>
       <c r="I55" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J55" s="101" t="s">
         <v>347</v>
@@ -4456,7 +4480,9 @@
       <c r="B57" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="C57" s="83"/>
+      <c r="C57" s="83" t="s">
+        <v>374</v>
+      </c>
       <c r="D57" s="83" t="s">
         <v>11</v>
       </c>
@@ -4466,10 +4492,14 @@
       <c r="F57" s="83" t="s">
         <v>371</v>
       </c>
-      <c r="G57" s="6"/>
-      <c r="H57" s="6"/>
+      <c r="G57" s="6">
+        <v>6.0999999999999999E-2</v>
+      </c>
+      <c r="H57" s="88">
+        <v>46205</v>
+      </c>
       <c r="I57" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J57" s="101" t="s">
         <v>347</v>
@@ -4538,7 +4568,9 @@
       <c r="B59" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="C59" s="83"/>
+      <c r="C59" s="83" t="s">
+        <v>373</v>
+      </c>
       <c r="D59" s="83" t="s">
         <v>11</v>
       </c>
@@ -4548,10 +4580,14 @@
       <c r="F59" s="83" t="s">
         <v>371</v>
       </c>
-      <c r="G59" s="6"/>
-      <c r="H59" s="6"/>
+      <c r="G59" s="6">
+        <v>8.2000000000000003E-2</v>
+      </c>
+      <c r="H59" s="88">
+        <v>46205</v>
+      </c>
       <c r="I59" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J59" s="101" t="s">
         <v>347</v>

</xml_diff>

<commit_message>
2 new meters installed
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1939" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60F1F77D-A634-4056-9D0A-68CE8D705D69}"/>
+  <xr:revisionPtr revIDLastSave="1947" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AB65D96-74F8-4021-BD23-1AD6229CAA95}"/>
   <bookViews>
     <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3050" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3052" uniqueCount="390">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -1202,6 +1202,9 @@
     <t>10192065</t>
   </si>
   <si>
+    <t>10192061</t>
+  </si>
+  <si>
     <t>9993239</t>
   </si>
   <si>
@@ -1209,6 +1212,9 @@
   </si>
   <si>
     <t>10192053</t>
+  </si>
+  <si>
+    <t>10192048</t>
   </si>
 </sst>
 </file>
@@ -3803,7 +3809,9 @@
       <c r="B39" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="C39" s="83"/>
+      <c r="C39" s="83" t="s">
+        <v>389</v>
+      </c>
       <c r="D39" s="83" t="s">
         <v>11</v>
       </c>
@@ -3813,10 +3821,14 @@
       <c r="F39" s="83" t="s">
         <v>371</v>
       </c>
-      <c r="G39" s="6"/>
-      <c r="H39" s="6"/>
+      <c r="G39" s="6">
+        <v>9.0999999999999998E-2</v>
+      </c>
+      <c r="H39" s="88">
+        <v>46205</v>
+      </c>
       <c r="I39" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J39" s="101" t="s">
         <v>348</v>
@@ -3885,7 +3897,9 @@
       <c r="B41" s="92" t="s">
         <v>10</v>
       </c>
-      <c r="C41" s="83"/>
+      <c r="C41" s="83" t="s">
+        <v>385</v>
+      </c>
       <c r="D41" s="83" t="s">
         <v>11</v>
       </c>
@@ -3895,10 +3909,14 @@
       <c r="F41" s="83" t="s">
         <v>371</v>
       </c>
-      <c r="G41" s="6"/>
-      <c r="H41" s="6"/>
+      <c r="G41" s="6">
+        <v>8.8999999999999996E-2</v>
+      </c>
+      <c r="H41" s="88">
+        <v>46205</v>
+      </c>
       <c r="I41" s="32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" s="101" t="s">
         <v>348</v>
@@ -3924,7 +3942,7 @@
         <v>16</v>
       </c>
       <c r="C42" s="83" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D42" s="83" t="s">
         <v>11</v>
@@ -4012,7 +4030,7 @@
         <v>16</v>
       </c>
       <c r="C44" s="83" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D44" s="83" t="s">
         <v>11</v>
@@ -4100,7 +4118,7 @@
         <v>16</v>
       </c>
       <c r="C46" s="83" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D46" s="83" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
New Water and Elec meters installed
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1955" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DFF3527-D3B8-4E96-A513-D55F04640F94}"/>
+  <xr:revisionPtr revIDLastSave="2029" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86204340-3AF9-440D-B5B6-96B8E5075F41}"/>
   <bookViews>
-    <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Water meters " sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3054" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3073" uniqueCount="395">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -1221,6 +1221,15 @@
   </si>
   <si>
     <t>9993262</t>
+  </si>
+  <si>
+    <t>10192010</t>
+  </si>
+  <si>
+    <t>10192016</t>
+  </si>
+  <si>
+    <t>9993259</t>
   </si>
 </sst>
 </file>
@@ -2051,10 +2060,6 @@
 </FeaturePropertyBags>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -6770,7 +6775,7 @@
         <v>127</v>
       </c>
       <c r="C106" s="83" t="s">
-        <v>146</v>
+        <v>392</v>
       </c>
       <c r="D106" s="83" t="s">
         <v>11</v>
@@ -6782,7 +6787,7 @@
         <v>371</v>
       </c>
       <c r="G106" s="6">
-        <v>9.2999999999999999E-2</v>
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="H106" s="88">
         <v>46168</v>
@@ -6934,7 +6939,7 @@
         <v>127</v>
       </c>
       <c r="C110" s="83" t="s">
-        <v>152</v>
+        <v>393</v>
       </c>
       <c r="D110" s="83" t="s">
         <v>11</v>
@@ -6946,7 +6951,7 @@
         <v>371</v>
       </c>
       <c r="G110" s="6">
-        <v>7.0999999999999994E-2</v>
+        <v>6.8000000000000005E-2</v>
       </c>
       <c r="H110" s="88">
         <v>46142</v>
@@ -7590,7 +7595,7 @@
         <v>127</v>
       </c>
       <c r="C126" s="83" t="s">
-        <v>176</v>
+        <v>394</v>
       </c>
       <c r="D126" s="83" t="s">
         <v>11</v>
@@ -7602,7 +7607,7 @@
         <v>371</v>
       </c>
       <c r="G126" s="6">
-        <v>1.163</v>
+        <v>9.0999999999999998E-2</v>
       </c>
       <c r="H126" s="88">
         <v>46168</v>
@@ -11887,7 +11892,9 @@
       <c r="B35" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C35" s="5"/>
+      <c r="C35" s="5">
+        <v>14558069275</v>
+      </c>
       <c r="D35" s="5">
         <v>82929684</v>
       </c>
@@ -11900,14 +11907,18 @@
       <c r="G35" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H35" s="5"/>
+      <c r="H35" s="16" t="s">
+        <v>278</v>
+      </c>
       <c r="I35" s="50" t="s">
         <v>295</v>
       </c>
       <c r="J35" s="18">
         <v>0</v>
       </c>
-      <c r="K35" s="5"/>
+      <c r="K35" s="13">
+        <v>46206</v>
+      </c>
       <c r="L35" s="20" t="b">
         <v>0</v>
       </c>
@@ -11934,7 +11945,9 @@
       <c r="B36" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C36" s="5"/>
+      <c r="C36" s="5">
+        <v>14558069325</v>
+      </c>
       <c r="D36" s="5">
         <v>82929684</v>
       </c>
@@ -11947,14 +11960,18 @@
       <c r="G36" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H36" s="5"/>
+      <c r="H36" s="17" t="s">
+        <v>277</v>
+      </c>
       <c r="I36" s="50" t="s">
         <v>295</v>
       </c>
       <c r="J36" s="18">
         <v>0</v>
       </c>
-      <c r="K36" s="5"/>
+      <c r="K36" s="13">
+        <v>46206</v>
+      </c>
       <c r="L36" s="20" t="b">
         <v>0</v>
       </c>
@@ -11981,7 +11998,9 @@
       <c r="B37" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C37" s="5"/>
+      <c r="C37" s="5">
+        <v>14558069978</v>
+      </c>
       <c r="D37" s="5">
         <v>82929684</v>
       </c>
@@ -11994,14 +12013,18 @@
       <c r="G37" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H37" s="5"/>
+      <c r="H37" s="5" t="s">
+        <v>275</v>
+      </c>
       <c r="I37" s="50" t="s">
         <v>295</v>
       </c>
       <c r="J37" s="18">
         <v>0</v>
       </c>
-      <c r="K37" s="5"/>
+      <c r="K37" s="13">
+        <v>46206</v>
+      </c>
       <c r="L37" s="20" t="b">
         <v>0</v>
       </c>
@@ -12028,7 +12051,9 @@
       <c r="B38" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C38" s="5"/>
+      <c r="C38" s="5">
+        <v>14558069283</v>
+      </c>
       <c r="D38" s="5">
         <v>82929684</v>
       </c>
@@ -12041,14 +12066,18 @@
       <c r="G38" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H38" s="5"/>
+      <c r="H38" s="16" t="s">
+        <v>278</v>
+      </c>
       <c r="I38" s="50" t="s">
         <v>295</v>
       </c>
       <c r="J38" s="18">
         <v>0</v>
       </c>
-      <c r="K38" s="5"/>
+      <c r="K38" s="13">
+        <v>46206</v>
+      </c>
       <c r="L38" s="20" t="b">
         <v>0</v>
       </c>
@@ -12075,7 +12104,9 @@
       <c r="B39" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C39" s="5"/>
+      <c r="C39" s="5">
+        <v>14558069473</v>
+      </c>
       <c r="D39" s="5">
         <v>82929684</v>
       </c>
@@ -12088,14 +12119,18 @@
       <c r="G39" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H39" s="5"/>
+      <c r="H39" s="16" t="s">
+        <v>278</v>
+      </c>
       <c r="I39" s="51" t="s">
         <v>297</v>
       </c>
       <c r="J39" s="18">
         <v>0</v>
       </c>
-      <c r="K39" s="5"/>
+      <c r="K39" s="13">
+        <v>46206</v>
+      </c>
       <c r="L39" s="20" t="b">
         <v>0</v>
       </c>
@@ -12122,7 +12157,9 @@
       <c r="B40" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C40" s="5"/>
+      <c r="C40" s="5">
+        <v>14558069366</v>
+      </c>
       <c r="D40" s="5">
         <v>82929684</v>
       </c>
@@ -12135,14 +12172,18 @@
       <c r="G40" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H40" s="5"/>
+      <c r="H40" s="5" t="s">
+        <v>275</v>
+      </c>
       <c r="I40" s="51" t="s">
         <v>297</v>
       </c>
       <c r="J40" s="18">
         <v>0</v>
       </c>
-      <c r="K40" s="5"/>
+      <c r="K40" s="13">
+        <v>46206</v>
+      </c>
       <c r="L40" s="20" t="b">
         <v>0</v>
       </c>
@@ -12169,7 +12210,9 @@
       <c r="B41" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C41" s="5"/>
+      <c r="C41" s="5">
+        <v>14558069614</v>
+      </c>
       <c r="D41" s="5">
         <v>82929684</v>
       </c>
@@ -12182,14 +12225,18 @@
       <c r="G41" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H41" s="5"/>
+      <c r="H41" s="5" t="s">
+        <v>275</v>
+      </c>
       <c r="I41" s="51" t="s">
         <v>297</v>
       </c>
       <c r="J41" s="18">
         <v>0</v>
       </c>
-      <c r="K41" s="5"/>
+      <c r="K41" s="13">
+        <v>46206</v>
+      </c>
       <c r="L41" s="20" t="b">
         <v>0</v>
       </c>
@@ -12216,7 +12263,9 @@
       <c r="B42" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C42" s="5"/>
+      <c r="C42" s="5">
+        <v>14558068905</v>
+      </c>
       <c r="D42" s="5">
         <v>82929684</v>
       </c>
@@ -12229,14 +12278,18 @@
       <c r="G42" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H42" s="5"/>
+      <c r="H42" s="17" t="s">
+        <v>277</v>
+      </c>
       <c r="I42" s="51" t="s">
         <v>297</v>
       </c>
       <c r="J42" s="18">
         <v>0</v>
       </c>
-      <c r="K42" s="5"/>
+      <c r="K42" s="13">
+        <v>46206</v>
+      </c>
       <c r="L42" s="20" t="b">
         <v>0</v>
       </c>
@@ -12263,7 +12316,9 @@
       <c r="B43" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C43" s="5"/>
+      <c r="C43" s="5">
+        <v>14558069630</v>
+      </c>
       <c r="D43" s="5">
         <v>82929684</v>
       </c>
@@ -12276,14 +12331,18 @@
       <c r="G43" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H43" s="5"/>
+      <c r="H43" s="17" t="s">
+        <v>277</v>
+      </c>
       <c r="I43" s="51" t="s">
         <v>297</v>
       </c>
       <c r="J43" s="18">
         <v>0</v>
       </c>
-      <c r="K43" s="5"/>
+      <c r="K43" s="13">
+        <v>46206</v>
+      </c>
       <c r="L43" s="20" t="b">
         <v>0</v>
       </c>
@@ -12310,7 +12369,9 @@
       <c r="B44" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C44" s="5"/>
+      <c r="C44" s="5">
+        <v>14558068863</v>
+      </c>
       <c r="D44" s="5">
         <v>82929684</v>
       </c>
@@ -12323,14 +12384,18 @@
       <c r="G44" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H44" s="5"/>
+      <c r="H44" s="16" t="s">
+        <v>278</v>
+      </c>
       <c r="I44" s="51" t="s">
         <v>297</v>
       </c>
       <c r="J44" s="18">
         <v>0</v>
       </c>
-      <c r="K44" s="5"/>
+      <c r="K44" s="13">
+        <v>46206</v>
+      </c>
       <c r="L44" s="20" t="b">
         <v>0</v>
       </c>
@@ -12357,7 +12422,9 @@
       <c r="B45" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C45" s="5"/>
+      <c r="C45" s="5">
+        <v>14558069655</v>
+      </c>
       <c r="D45" s="5">
         <v>82929684</v>
       </c>
@@ -12370,14 +12437,18 @@
       <c r="G45" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H45" s="5"/>
+      <c r="H45" s="16" t="s">
+        <v>278</v>
+      </c>
       <c r="I45" s="51" t="s">
         <v>297</v>
       </c>
       <c r="J45" s="18">
         <v>0</v>
       </c>
-      <c r="K45" s="5"/>
+      <c r="K45" s="13">
+        <v>46206</v>
+      </c>
       <c r="L45" s="20" t="b">
         <v>0</v>
       </c>
@@ -12404,7 +12475,9 @@
       <c r="B46" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C46" s="5"/>
+      <c r="C46" s="5">
+        <v>14558069622</v>
+      </c>
       <c r="D46" s="5">
         <v>82929684</v>
       </c>
@@ -12417,14 +12490,18 @@
       <c r="G46" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H46" s="5"/>
+      <c r="H46" s="5" t="s">
+        <v>275</v>
+      </c>
       <c r="I46" s="51" t="s">
         <v>297</v>
       </c>
       <c r="J46" s="18">
         <v>0</v>
       </c>
-      <c r="K46" s="5"/>
+      <c r="K46" s="13">
+        <v>46206</v>
+      </c>
       <c r="L46" s="20" t="b">
         <v>0</v>
       </c>
@@ -12733,7 +12810,9 @@
       <c r="B53" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C53" s="5"/>
+      <c r="C53" s="5">
+        <v>14558069895</v>
+      </c>
       <c r="D53" s="5">
         <v>82929684</v>
       </c>
@@ -12746,14 +12825,18 @@
       <c r="G53" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H53" s="5"/>
+      <c r="H53" s="5" t="s">
+        <v>275</v>
+      </c>
       <c r="I53" s="39" t="s">
         <v>289</v>
       </c>
       <c r="J53" s="18">
         <v>0</v>
       </c>
-      <c r="K53" s="5"/>
+      <c r="K53" s="13">
+        <v>46206</v>
+      </c>
       <c r="L53" s="20" t="b">
         <v>0</v>
       </c>
@@ -12780,7 +12863,9 @@
       <c r="B54" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C54" s="5"/>
+      <c r="C54" s="5">
+        <v>14558069192</v>
+      </c>
       <c r="D54" s="5">
         <v>82929684</v>
       </c>
@@ -12793,14 +12878,18 @@
       <c r="G54" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H54" s="5"/>
+      <c r="H54" s="16" t="s">
+        <v>278</v>
+      </c>
       <c r="I54" s="39" t="s">
         <v>289</v>
       </c>
       <c r="J54" s="18">
         <v>0</v>
       </c>
-      <c r="K54" s="5"/>
+      <c r="K54" s="13">
+        <v>46206</v>
+      </c>
       <c r="L54" s="20" t="b">
         <v>0</v>
       </c>
@@ -12827,7 +12916,9 @@
       <c r="B55" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C55" s="5"/>
+      <c r="C55" s="5">
+        <v>14558068269</v>
+      </c>
       <c r="D55" s="5">
         <v>82929684</v>
       </c>
@@ -12840,14 +12931,18 @@
       <c r="G55" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H55" s="5"/>
+      <c r="H55" s="16" t="s">
+        <v>278</v>
+      </c>
       <c r="I55" s="39" t="s">
         <v>289</v>
       </c>
       <c r="J55" s="18">
         <v>0</v>
       </c>
-      <c r="K55" s="5"/>
+      <c r="K55" s="13">
+        <v>46206</v>
+      </c>
       <c r="L55" s="20" t="b">
         <v>0</v>
       </c>
@@ -12874,7 +12969,9 @@
       <c r="B56" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C56" s="5"/>
+      <c r="C56" s="5">
+        <v>14558068426</v>
+      </c>
       <c r="D56" s="5">
         <v>82929684</v>
       </c>
@@ -12887,14 +12984,18 @@
       <c r="G56" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H56" s="5"/>
+      <c r="H56" s="5" t="s">
+        <v>275</v>
+      </c>
       <c r="I56" s="39" t="s">
         <v>289</v>
       </c>
       <c r="J56" s="18">
         <v>0</v>
       </c>
-      <c r="K56" s="5"/>
+      <c r="K56" s="13">
+        <v>46206</v>
+      </c>
       <c r="L56" s="20" t="b">
         <v>0</v>
       </c>
@@ -12921,7 +13022,9 @@
       <c r="B57" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C57" s="5"/>
+      <c r="C57" s="5">
+        <v>14558069358</v>
+      </c>
       <c r="D57" s="5">
         <v>82929684</v>
       </c>
@@ -12934,14 +13037,18 @@
       <c r="G57" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H57" s="5"/>
+      <c r="H57" s="17" t="s">
+        <v>277</v>
+      </c>
       <c r="I57" s="39" t="s">
         <v>289</v>
       </c>
       <c r="J57" s="18">
         <v>0</v>
       </c>
-      <c r="K57" s="5"/>
+      <c r="K57" s="13">
+        <v>46206</v>
+      </c>
       <c r="L57" s="20" t="b">
         <v>0</v>
       </c>
@@ -12968,7 +13075,9 @@
       <c r="B58" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C58" s="5"/>
+      <c r="C58" s="5">
+        <v>14558068327</v>
+      </c>
       <c r="D58" s="5">
         <v>82929684</v>
       </c>
@@ -12981,14 +13090,18 @@
       <c r="G58" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H58" s="5"/>
+      <c r="H58" s="17" t="s">
+        <v>277</v>
+      </c>
       <c r="I58" s="39" t="s">
         <v>289</v>
       </c>
       <c r="J58" s="18">
         <v>0</v>
       </c>
-      <c r="K58" s="5"/>
+      <c r="K58" s="13">
+        <v>46206</v>
+      </c>
       <c r="L58" s="20" t="b">
         <v>0</v>
       </c>
@@ -13068,7 +13181,9 @@
       <c r="B60" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C60" s="5"/>
+      <c r="C60" s="5">
+        <v>14558069531</v>
+      </c>
       <c r="D60" s="5">
         <v>82929684</v>
       </c>
@@ -13081,14 +13196,18 @@
       <c r="G60" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H60" s="5"/>
+      <c r="H60" s="16" t="s">
+        <v>278</v>
+      </c>
       <c r="I60" s="39" t="s">
         <v>289</v>
       </c>
       <c r="J60" s="18">
         <v>0</v>
       </c>
-      <c r="K60" s="5"/>
+      <c r="K60" s="13">
+        <v>46206</v>
+      </c>
       <c r="L60" s="20" t="b">
         <v>0</v>
       </c>
@@ -21030,10 +21149,12 @@
       <c r="D4" s="7">
         <v>17968.5</v>
       </c>
-      <c r="E4" s="6"/>
+      <c r="E4" s="6">
+        <v>18120.900000000001</v>
+      </c>
       <c r="F4" s="6">
         <f t="shared" si="0"/>
-        <v>-17968.5</v>
+        <v>152.40000000000146</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">

</xml_diff>

<commit_message>
Meter replacement dates inserted
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2148" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5AAA1884-9E91-478E-9800-06D5D126536A}"/>
+  <xr:revisionPtr revIDLastSave="2159" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C542235-3299-4716-A8F3-4093F730D3CB}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Water meters " sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Elec Meters'!$A$1:$Q$192</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Water meters '!$A$1:$N$193</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Water meters '!$A$1:$Q$193</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -1597,7 +1597,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1892,17 +1892,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2338,7 +2335,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q193"/>
+  <dimension ref="A1:Q204"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
@@ -2349,9 +2346,9 @@
     <col min="10" max="10" width="27.3984375" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="20.19921875" customWidth="1"/>
     <col min="14" max="14" width="35.53125" customWidth="1"/>
-    <col min="15" max="15" width="14.33203125" customWidth="1"/>
-    <col min="16" max="16" width="17.3984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.1328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.06640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="25.9296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="29.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="18" x14ac:dyDescent="0.3">
@@ -2397,13 +2394,13 @@
       <c r="N1" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="O1" s="100" t="s">
+      <c r="O1" s="98" t="s">
         <v>394</v>
       </c>
-      <c r="P1" s="100" t="s">
+      <c r="P1" s="98" t="s">
         <v>395</v>
       </c>
-      <c r="Q1" s="101" t="s">
+      <c r="Q1" s="1" t="s">
         <v>396</v>
       </c>
     </row>
@@ -7556,7 +7553,9 @@
       <c r="P106" s="23" t="b">
         <v>1</v>
       </c>
-      <c r="Q106" s="19"/>
+      <c r="Q106" s="78">
+        <v>46206</v>
+      </c>
     </row>
     <row r="107" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
       <c r="A107" s="25" t="s">
@@ -7748,7 +7747,9 @@
       <c r="P110" s="23" t="b">
         <v>1</v>
       </c>
-      <c r="Q110" s="19"/>
+      <c r="Q110" s="78">
+        <v>46206</v>
+      </c>
     </row>
     <row r="111" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
       <c r="A111" s="25" t="s">
@@ -8516,7 +8517,9 @@
       <c r="P126" s="23" t="b">
         <v>1</v>
       </c>
-      <c r="Q126" s="19"/>
+      <c r="Q126" s="78">
+        <v>46206</v>
+      </c>
     </row>
     <row r="127" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
       <c r="A127" s="25" t="s">
@@ -11598,6 +11601,11 @@
         <v>0</v>
       </c>
       <c r="Q193" s="19"/>
+    </row>
+    <row r="204" spans="1:17" ht="18" x14ac:dyDescent="0.3">
+      <c r="Q204" s="78">
+        <v>46206</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N193">
@@ -21420,34 +21428,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="14.65" x14ac:dyDescent="0.45">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="99" t="s">
         <v>303</v>
       </c>
-      <c r="B1" s="98" t="s">
+      <c r="B1" s="99" t="s">
         <v>304</v>
       </c>
-      <c r="C1" s="98" t="s">
+      <c r="C1" s="99" t="s">
         <v>305</v>
       </c>
-      <c r="D1" s="99" t="s">
+      <c r="D1" s="100" t="s">
         <v>306</v>
       </c>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99" t="s">
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100" t="s">
         <v>307</v>
       </c>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
+      <c r="H1" s="100"/>
+      <c r="I1" s="100"/>
       <c r="J1" s="19"/>
       <c r="K1" s="67" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="14.65" x14ac:dyDescent="0.45">
-      <c r="A2" s="98"/>
-      <c r="B2" s="98"/>
-      <c r="C2" s="98"/>
+      <c r="A2" s="99"/>
+      <c r="B2" s="99"/>
+      <c r="C2" s="99"/>
       <c r="D2" s="18" t="s">
         <v>308</v>
       </c>
@@ -23702,19 +23710,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="14.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="99" t="s">
         <v>325</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="98"/>
-      <c r="D1" s="98"/>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="98"/>
-      <c r="H1" s="98"/>
-      <c r="I1" s="98"/>
-      <c r="J1" s="98"/>
-      <c r="K1" s="98"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
+      <c r="H1" s="99"/>
+      <c r="I1" s="99"/>
+      <c r="J1" s="99"/>
+      <c r="K1" s="99"/>
     </row>
     <row r="2" spans="1:11" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
@@ -24447,16 +24455,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="99" t="s">
         <v>326</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="98"/>
-      <c r="D1" s="98"/>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="98"/>
-      <c r="H1" s="98"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
+      <c r="H1" s="99"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">

</xml_diff>

<commit_message>
New meters replaced and meter serial updates
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2235" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F09BE78-4057-413F-ABEA-F21BBAD87E41}"/>
+  <xr:revisionPtr revIDLastSave="2246" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF516590-4E44-4B9A-9CEB-F6D696FF7B22}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FS Elec" sheetId="4" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4966" uniqueCount="1190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4967" uniqueCount="1192">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -3617,6 +3617,12 @@
   </si>
   <si>
     <t>MS3</t>
+  </si>
+  <si>
+    <t>9993247</t>
+  </si>
+  <si>
+    <t>10192047</t>
   </si>
 </sst>
 </file>
@@ -19628,8 +19634,8 @@
       <c r="B97" s="79" t="s">
         <v>119</v>
       </c>
-      <c r="C97" s="73">
-        <v>10172132</v>
+      <c r="C97" s="73" t="s">
+        <v>1190</v>
       </c>
       <c r="D97" s="73" t="s">
         <v>11</v>
@@ -19668,9 +19674,11 @@
         <v>1</v>
       </c>
       <c r="P97" s="23" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q97" s="19"/>
+        <v>1</v>
+      </c>
+      <c r="Q97" s="78">
+        <v>46216</v>
+      </c>
     </row>
     <row r="98" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
       <c r="A98" s="25" t="s">
@@ -19692,7 +19700,7 @@
         <v>369</v>
       </c>
       <c r="G98" s="3">
-        <v>9.9000000000000005E-2</v>
+        <v>8.2000000000000003E-2</v>
       </c>
       <c r="H98" s="78">
         <v>46168</v>
@@ -19986,7 +19994,7 @@
         <v>127</v>
       </c>
       <c r="C104" s="73" t="s">
-        <v>143</v>
+        <v>1191</v>
       </c>
       <c r="D104" s="73" t="s">
         <v>11</v>
@@ -19998,7 +20006,7 @@
         <v>369</v>
       </c>
       <c r="G104" s="3">
-        <v>7.2999999999999995E-2</v>
+        <v>9.7000000000000003E-2</v>
       </c>
       <c r="H104" s="78">
         <v>46168</v>
@@ -20025,9 +20033,11 @@
         <v>1</v>
       </c>
       <c r="P104" s="23" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q104" s="19"/>
+        <v>1</v>
+      </c>
+      <c r="Q104" s="78">
+        <v>46216</v>
+      </c>
     </row>
     <row r="105" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
       <c r="A105" s="25" t="s">
@@ -24614,7 +24624,7 @@
         <v>690</v>
       </c>
       <c r="C21" s="100">
-        <v>87818204</v>
+        <v>87819204</v>
       </c>
       <c r="D21" s="103">
         <v>87818877</v>
@@ -27954,7 +27964,7 @@
         <v>846</v>
       </c>
       <c r="C188" s="100">
-        <v>90008072</v>
+        <v>90008082</v>
       </c>
       <c r="D188" s="101">
         <v>83013891</v>

</xml_diff>

<commit_message>
new meter removals and replacements
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2356" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9A5DA56-4CD4-46C6-AAD7-235815223520}"/>
+  <xr:revisionPtr revIDLastSave="2357" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4F478B0-D9EA-4E2A-BD15-2B5C94F123DB}"/>
   <bookViews>
     <workbookView xWindow="43080" yWindow="-2565" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19937,7 +19937,7 @@
         <v>46168</v>
       </c>
       <c r="O95" s="21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P95" s="21" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
NEw electrical meters and AMR installed update list
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2444" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A47FEE63-9793-4298-864B-BEC6537C68C4}"/>
+  <xr:revisionPtr revIDLastSave="2575" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C5BF501-A530-4B8C-A6AB-77A70641A1B2}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-2565" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="21720" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FS Elec" sheetId="4" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4987" uniqueCount="1193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5000" uniqueCount="1194">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -3626,6 +3626,9 @@
   </si>
   <si>
     <t>10192062</t>
+  </si>
+  <si>
+    <t xml:space="preserve">removal date </t>
   </si>
 </sst>
 </file>
@@ -4248,7 +4251,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="37" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="162">
+  <cellXfs count="164">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4735,6 +4738,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5755,7 +5764,9 @@
       <c r="B11" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="2">
+        <v>14558066248</v>
+      </c>
       <c r="D11" s="2">
         <v>82929702</v>
       </c>
@@ -5768,14 +5779,18 @@
       <c r="G11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="2"/>
+      <c r="H11" s="7" t="s">
+        <v>64</v>
+      </c>
       <c r="I11" s="46" t="s">
         <v>35</v>
       </c>
       <c r="J11" s="9">
         <v>0</v>
       </c>
-      <c r="K11" s="2"/>
+      <c r="K11" s="4">
+        <v>46218</v>
+      </c>
       <c r="L11" s="11" t="b">
         <v>0</v>
       </c>
@@ -5803,7 +5818,9 @@
       <c r="B12" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="2">
+        <v>14558069416</v>
+      </c>
       <c r="D12" s="2">
         <v>82929702</v>
       </c>
@@ -5816,14 +5833,18 @@
       <c r="G12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H12" s="2"/>
+      <c r="H12" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="I12" s="46" t="s">
         <v>35</v>
       </c>
       <c r="J12" s="9">
         <v>0</v>
       </c>
-      <c r="K12" s="2"/>
+      <c r="K12" s="4">
+        <v>46218</v>
+      </c>
       <c r="L12" s="11" t="b">
         <v>0</v>
       </c>
@@ -5851,7 +5872,9 @@
       <c r="B13" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="2"/>
+      <c r="C13" s="2">
+        <v>14558069465</v>
+      </c>
       <c r="D13" s="2">
         <v>82929702</v>
       </c>
@@ -5864,14 +5887,18 @@
       <c r="G13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H13" s="2"/>
+      <c r="H13" s="7" t="s">
+        <v>64</v>
+      </c>
       <c r="I13" s="46" t="s">
         <v>35</v>
       </c>
       <c r="J13" s="9">
         <v>0</v>
       </c>
-      <c r="K13" s="2"/>
+      <c r="K13" s="4">
+        <v>46218</v>
+      </c>
       <c r="L13" s="11" t="b">
         <v>0</v>
       </c>
@@ -5947,7 +5974,9 @@
       <c r="B15" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="2"/>
+      <c r="C15" s="2">
+        <v>14558066305</v>
+      </c>
       <c r="D15" s="2">
         <v>82929702</v>
       </c>
@@ -5960,14 +5989,18 @@
       <c r="G15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H15" s="2"/>
+      <c r="H15" s="7" t="s">
+        <v>64</v>
+      </c>
       <c r="I15" s="46" t="s">
         <v>35</v>
       </c>
       <c r="J15" s="9">
         <v>0</v>
       </c>
-      <c r="K15" s="2"/>
+      <c r="K15" s="4">
+        <v>46218</v>
+      </c>
       <c r="L15" s="11" t="b">
         <v>0</v>
       </c>
@@ -6043,7 +6076,9 @@
       <c r="B17" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="2"/>
+      <c r="C17" s="2">
+        <v>14558068939</v>
+      </c>
       <c r="D17" s="2">
         <v>82929702</v>
       </c>
@@ -6056,14 +6091,18 @@
       <c r="G17" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H17" s="2"/>
+      <c r="H17" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="I17" s="46" t="s">
         <v>35</v>
       </c>
       <c r="J17" s="9">
         <v>0</v>
       </c>
-      <c r="K17" s="2"/>
+      <c r="K17" s="4">
+        <v>46218</v>
+      </c>
       <c r="L17" s="11" t="b">
         <v>0</v>
       </c>
@@ -6139,7 +6178,9 @@
       <c r="B19" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="2"/>
+      <c r="C19" s="2">
+        <v>14558066099</v>
+      </c>
       <c r="D19" s="2">
         <v>82929702</v>
       </c>
@@ -6152,14 +6193,18 @@
       <c r="G19" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H19" s="2"/>
+      <c r="H19" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="I19" s="46" t="s">
         <v>35</v>
       </c>
       <c r="J19" s="9">
         <v>0</v>
       </c>
-      <c r="K19" s="2"/>
+      <c r="K19" s="4">
+        <v>46218</v>
+      </c>
       <c r="L19" s="11" t="b">
         <v>0</v>
       </c>
@@ -6187,7 +6232,9 @@
       <c r="B20" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="2"/>
+      <c r="C20" s="2">
+        <v>14558069481</v>
+      </c>
       <c r="D20" s="2">
         <v>82929702</v>
       </c>
@@ -6200,14 +6247,18 @@
       <c r="G20" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H20" s="2"/>
+      <c r="H20" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="I20" s="40" t="s">
         <v>46</v>
       </c>
       <c r="J20" s="9">
         <v>0</v>
       </c>
-      <c r="K20" s="2"/>
+      <c r="K20" s="4">
+        <v>46218</v>
+      </c>
       <c r="L20" s="11" t="b">
         <v>0</v>
       </c>
@@ -6235,7 +6286,9 @@
       <c r="B21" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C21" s="2"/>
+      <c r="C21" s="2">
+        <v>14558068434</v>
+      </c>
       <c r="D21" s="2">
         <v>82929702</v>
       </c>
@@ -6248,14 +6301,18 @@
       <c r="G21" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H21" s="2"/>
+      <c r="H21" s="7" t="s">
+        <v>64</v>
+      </c>
       <c r="I21" s="40" t="s">
         <v>46</v>
       </c>
       <c r="J21" s="9">
         <v>0</v>
       </c>
-      <c r="K21" s="2"/>
+      <c r="K21" s="4">
+        <v>46218</v>
+      </c>
       <c r="L21" s="11" t="b">
         <v>0</v>
       </c>
@@ -6283,7 +6340,9 @@
       <c r="B22" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="2"/>
+      <c r="C22" s="2">
+        <v>14558068798</v>
+      </c>
       <c r="D22" s="2">
         <v>82929702</v>
       </c>
@@ -6296,14 +6355,18 @@
       <c r="G22" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H22" s="2"/>
+      <c r="H22" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="I22" s="40" t="s">
         <v>46</v>
       </c>
       <c r="J22" s="9">
         <v>0</v>
       </c>
-      <c r="K22" s="2"/>
+      <c r="K22" s="4">
+        <v>46218</v>
+      </c>
       <c r="L22" s="11" t="b">
         <v>0</v>
       </c>
@@ -6331,7 +6394,9 @@
       <c r="B23" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="2"/>
+      <c r="C23" s="2">
+        <v>14558069002</v>
+      </c>
       <c r="D23" s="2">
         <v>82929702</v>
       </c>
@@ -6344,14 +6409,18 @@
       <c r="G23" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H23" s="2"/>
+      <c r="H23" s="7" t="s">
+        <v>64</v>
+      </c>
       <c r="I23" s="40" t="s">
         <v>46</v>
       </c>
       <c r="J23" s="9">
         <v>0</v>
       </c>
-      <c r="K23" s="2"/>
+      <c r="K23" s="4">
+        <v>46218</v>
+      </c>
       <c r="L23" s="11" t="b">
         <v>0</v>
       </c>
@@ -6379,7 +6448,9 @@
       <c r="B24" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="2"/>
+      <c r="C24" s="163">
+        <v>14558068921</v>
+      </c>
       <c r="D24" s="2">
         <v>82929702</v>
       </c>
@@ -6392,14 +6463,18 @@
       <c r="G24" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H24" s="2"/>
+      <c r="H24" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="I24" s="40" t="s">
         <v>46</v>
       </c>
       <c r="J24" s="9">
         <v>0</v>
       </c>
-      <c r="K24" s="2"/>
+      <c r="K24" s="4">
+        <v>46218</v>
+      </c>
       <c r="L24" s="11" t="b">
         <v>0</v>
       </c>
@@ -6427,7 +6502,9 @@
       <c r="B25" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="2"/>
+      <c r="C25" s="2">
+        <v>14558069374</v>
+      </c>
       <c r="D25" s="2">
         <v>82929702</v>
       </c>
@@ -6440,14 +6517,18 @@
       <c r="G25" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H25" s="2"/>
+      <c r="H25" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="I25" s="40" t="s">
         <v>46</v>
       </c>
       <c r="J25" s="9">
         <v>0</v>
       </c>
-      <c r="K25" s="2"/>
+      <c r="K25" s="4">
+        <v>46218</v>
+      </c>
       <c r="L25" s="11" t="b">
         <v>0</v>
       </c>
@@ -8827,7 +8908,9 @@
       <c r="L69" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M69" s="2"/>
+      <c r="M69" s="2">
+        <v>6</v>
+      </c>
       <c r="N69" s="64" t="s">
         <v>105</v>
       </c>
@@ -8879,9 +8962,11 @@
         <v>46197</v>
       </c>
       <c r="L70" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M70" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M70" s="2">
+        <v>5</v>
+      </c>
       <c r="N70" s="64" t="s">
         <v>103</v>
       </c>
@@ -8935,7 +9020,9 @@
       <c r="L71" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M71" s="2"/>
+      <c r="M71" s="2">
+        <v>7</v>
+      </c>
       <c r="N71" s="64" t="s">
         <v>105</v>
       </c>
@@ -8987,9 +9074,11 @@
         <v>46197</v>
       </c>
       <c r="L72" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M72" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M72" s="2">
+        <v>1</v>
+      </c>
       <c r="N72" s="64" t="s">
         <v>103</v>
       </c>
@@ -9041,9 +9130,11 @@
         <v>46197</v>
       </c>
       <c r="L73" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M73" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M73" s="2">
+        <v>8</v>
+      </c>
       <c r="N73" s="64" t="s">
         <v>105</v>
       </c>
@@ -9097,7 +9188,9 @@
       <c r="L74" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M74" s="2"/>
+      <c r="M74" s="2">
+        <v>2</v>
+      </c>
       <c r="N74" s="64" t="s">
         <v>103</v>
       </c>
@@ -9149,9 +9242,11 @@
         <v>46197</v>
       </c>
       <c r="L75" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M75" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M75" s="2">
+        <v>4</v>
+      </c>
       <c r="N75" s="64" t="s">
         <v>105</v>
       </c>
@@ -9203,9 +9298,11 @@
         <v>46197</v>
       </c>
       <c r="L76" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M76" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M76" s="2">
+        <v>3</v>
+      </c>
       <c r="N76" s="64" t="s">
         <v>103</v>
       </c>
@@ -14523,7 +14620,9 @@
       <c r="L177" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M177" s="2"/>
+      <c r="M177" s="2">
+        <v>1</v>
+      </c>
       <c r="N177" s="64" t="s">
         <v>250</v>
       </c>
@@ -14577,7 +14676,9 @@
       <c r="L178" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M178" s="2"/>
+      <c r="M178" s="2">
+        <v>2</v>
+      </c>
       <c r="N178" s="64" t="s">
         <v>250</v>
       </c>
@@ -14631,7 +14732,9 @@
       <c r="L179" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M179" s="2"/>
+      <c r="M179" s="2">
+        <v>3</v>
+      </c>
       <c r="N179" s="64" t="s">
         <v>250</v>
       </c>
@@ -14683,9 +14786,11 @@
         <v>46210</v>
       </c>
       <c r="L180" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M180" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M180" s="2">
+        <v>4</v>
+      </c>
       <c r="N180" s="64" t="s">
         <v>250</v>
       </c>
@@ -14739,7 +14844,9 @@
       <c r="L181" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M181" s="2"/>
+      <c r="M181" s="2">
+        <v>5</v>
+      </c>
       <c r="N181" s="64" t="s">
         <v>250</v>
       </c>
@@ -14793,7 +14900,9 @@
       <c r="L182" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M182" s="2"/>
+      <c r="M182" s="2">
+        <v>6</v>
+      </c>
       <c r="N182" s="64" t="s">
         <v>250</v>
       </c>
@@ -14847,7 +14956,9 @@
       <c r="L183" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M183" s="2"/>
+      <c r="M183" s="2">
+        <v>1</v>
+      </c>
       <c r="N183" s="64" t="s">
         <v>250</v>
       </c>
@@ -14901,7 +15012,9 @@
       <c r="L184" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M184" s="2"/>
+      <c r="M184" s="2">
+        <v>2</v>
+      </c>
       <c r="N184" s="64" t="s">
         <v>261</v>
       </c>
@@ -14955,7 +15068,9 @@
       <c r="L185" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M185" s="2"/>
+      <c r="M185" s="2">
+        <v>3</v>
+      </c>
       <c r="N185" s="64" t="s">
         <v>261</v>
       </c>
@@ -15009,7 +15124,9 @@
       <c r="L186" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M186" s="2"/>
+      <c r="M186" s="2">
+        <v>4</v>
+      </c>
       <c r="N186" s="64" t="s">
         <v>261</v>
       </c>
@@ -15061,9 +15178,11 @@
         <v>46210</v>
       </c>
       <c r="L187" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M187" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M187" s="2">
+        <v>5</v>
+      </c>
       <c r="N187" s="64" t="s">
         <v>261</v>
       </c>
@@ -15115,9 +15234,11 @@
         <v>46210</v>
       </c>
       <c r="L188" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M188" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M188" s="2">
+        <v>6</v>
+      </c>
       <c r="N188" s="64" t="s">
         <v>261</v>
       </c>
@@ -15361,7 +15482,7 @@
     <sortCondition ref="A2:A192"/>
   </sortState>
   <phoneticPr fontId="8" type="noConversion"/>
-  <conditionalFormatting sqref="C2:C192">
+  <conditionalFormatting sqref="C25:C192 C2:C23">
     <cfRule type="duplicateValues" dxfId="16" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C117:C122">
@@ -18406,7 +18527,7 @@
         <v>46195</v>
       </c>
       <c r="O63" s="21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P63" s="21" t="b">
         <v>0</v>
@@ -35864,20 +35985,20 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.73046875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.265625" customWidth="1"/>
     <col min="3" max="3" width="25.265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.1328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.86328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.3984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="127" t="s">
         <v>1178</v>
       </c>
@@ -35894,16 +36015,19 @@
         <v>1179</v>
       </c>
       <c r="F1" s="129" t="s">
+        <v>1193</v>
+      </c>
+      <c r="G1" s="129" t="s">
         <v>1180</v>
       </c>
-      <c r="G1" s="129" t="s">
+      <c r="H1" s="129" t="s">
         <v>1181</v>
       </c>
-      <c r="H1" s="105" t="s">
+      <c r="I1" s="105" t="s">
         <v>1179</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A2" s="130">
         <v>22</v>
       </c>
@@ -35917,14 +36041,19 @@
         <v>19375.900000000001</v>
       </c>
       <c r="E2" s="130"/>
-      <c r="F2" s="130"/>
-      <c r="G2" s="131">
-        <f t="shared" ref="G2:G34" si="0">F2-D2</f>
-        <v>-19375.900000000001</v>
-      </c>
-      <c r="H2" s="106"/>
-    </row>
-    <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="F2" s="162">
+        <v>46218</v>
+      </c>
+      <c r="G2" s="130">
+        <v>19888.099999999999</v>
+      </c>
+      <c r="H2" s="131">
+        <f t="shared" ref="H2:H34" si="0">G2-D2</f>
+        <v>512.19999999999709</v>
+      </c>
+      <c r="I2" s="106"/>
+    </row>
+    <row r="3" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A3" s="130">
         <v>44</v>
       </c>
@@ -35938,16 +36067,17 @@
         <v>56032.6</v>
       </c>
       <c r="E3" s="130"/>
-      <c r="F3" s="130">
+      <c r="F3" s="162"/>
+      <c r="G3" s="130">
         <v>56111.5</v>
       </c>
-      <c r="G3" s="131">
+      <c r="H3" s="131">
         <f t="shared" si="0"/>
         <v>78.900000000001455</v>
       </c>
-      <c r="H3" s="106"/>
-    </row>
-    <row r="4" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I3" s="106"/>
+    </row>
+    <row r="4" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A4" s="130">
         <v>53</v>
       </c>
@@ -35961,16 +36091,17 @@
         <v>17968.5</v>
       </c>
       <c r="E4" s="130"/>
-      <c r="F4" s="130">
+      <c r="F4" s="162"/>
+      <c r="G4" s="130">
         <v>18120.900000000001</v>
       </c>
-      <c r="G4" s="131">
+      <c r="H4" s="131">
         <f t="shared" si="0"/>
         <v>152.40000000000146</v>
       </c>
-      <c r="H4" s="106"/>
-    </row>
-    <row r="5" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I4" s="106"/>
+    </row>
+    <row r="5" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A5" s="132">
         <v>58</v>
       </c>
@@ -35984,16 +36115,17 @@
         <v>59659</v>
       </c>
       <c r="E5" s="132"/>
-      <c r="F5" s="130">
+      <c r="F5" s="162"/>
+      <c r="G5" s="130">
         <v>59659</v>
       </c>
-      <c r="G5" s="131">
+      <c r="H5" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H5" s="106"/>
-    </row>
-    <row r="6" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I5" s="106"/>
+    </row>
+    <row r="6" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A6" s="132">
         <v>60</v>
       </c>
@@ -36007,16 +36139,17 @@
         <v>97390</v>
       </c>
       <c r="E6" s="132"/>
-      <c r="F6" s="130">
+      <c r="F6" s="162"/>
+      <c r="G6" s="130">
         <v>97390</v>
       </c>
-      <c r="G6" s="131">
+      <c r="H6" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="106"/>
-    </row>
-    <row r="7" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I6" s="106"/>
+    </row>
+    <row r="7" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A7" s="132">
         <v>61</v>
       </c>
@@ -36030,16 +36163,17 @@
         <v>23184</v>
       </c>
       <c r="E7" s="132"/>
-      <c r="F7" s="130">
+      <c r="F7" s="162"/>
+      <c r="G7" s="130">
         <v>23184</v>
       </c>
-      <c r="G7" s="131">
+      <c r="H7" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H7" s="106"/>
-    </row>
-    <row r="8" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I7" s="106"/>
+    </row>
+    <row r="8" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A8" s="132">
         <v>62</v>
       </c>
@@ -36053,16 +36187,17 @@
         <v>7889</v>
       </c>
       <c r="E8" s="132"/>
-      <c r="F8" s="130">
+      <c r="F8" s="162"/>
+      <c r="G8" s="130">
         <v>7889</v>
       </c>
-      <c r="G8" s="131">
+      <c r="H8" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="106"/>
-    </row>
-    <row r="9" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I8" s="106"/>
+    </row>
+    <row r="9" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A9" s="132">
         <v>63</v>
       </c>
@@ -36076,16 +36211,17 @@
         <v>27096</v>
       </c>
       <c r="E9" s="132"/>
-      <c r="F9" s="130">
+      <c r="F9" s="162"/>
+      <c r="G9" s="130">
         <v>27095</v>
       </c>
-      <c r="G9" s="131">
+      <c r="H9" s="131">
         <f t="shared" si="0"/>
         <v>-1</v>
       </c>
-      <c r="H9" s="106"/>
-    </row>
-    <row r="10" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I9" s="106"/>
+    </row>
+    <row r="10" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A10" s="132">
         <v>64</v>
       </c>
@@ -36099,16 +36235,17 @@
         <v>15280</v>
       </c>
       <c r="E10" s="132"/>
-      <c r="F10" s="130">
+      <c r="F10" s="162"/>
+      <c r="G10" s="130">
         <v>15280</v>
       </c>
-      <c r="G10" s="131">
+      <c r="H10" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="106"/>
-    </row>
-    <row r="11" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I10" s="106"/>
+    </row>
+    <row r="11" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A11" s="132">
         <v>65</v>
       </c>
@@ -36122,16 +36259,17 @@
         <v>20310</v>
       </c>
       <c r="E11" s="132"/>
-      <c r="F11" s="130">
+      <c r="F11" s="162"/>
+      <c r="G11" s="130">
         <v>20310</v>
       </c>
-      <c r="G11" s="131">
+      <c r="H11" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H11" s="106"/>
-    </row>
-    <row r="12" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I11" s="106"/>
+    </row>
+    <row r="12" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A12" s="132">
         <v>66</v>
       </c>
@@ -36145,16 +36283,17 @@
         <v>24100</v>
       </c>
       <c r="E12" s="132"/>
-      <c r="F12" s="130">
+      <c r="F12" s="162"/>
+      <c r="G12" s="130">
         <v>24100</v>
       </c>
-      <c r="G12" s="131">
+      <c r="H12" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="106"/>
-    </row>
-    <row r="13" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I12" s="106"/>
+    </row>
+    <row r="13" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A13" s="132">
         <v>67</v>
       </c>
@@ -36168,16 +36307,17 @@
         <v>172161.6</v>
       </c>
       <c r="E13" s="132"/>
-      <c r="F13" s="130">
+      <c r="F13" s="162"/>
+      <c r="G13" s="130">
         <v>172161.6</v>
       </c>
-      <c r="G13" s="131">
+      <c r="H13" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H13" s="106"/>
-    </row>
-    <row r="14" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I13" s="106"/>
+    </row>
+    <row r="14" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A14" s="132">
         <v>68</v>
       </c>
@@ -36191,16 +36331,17 @@
         <v>11718</v>
       </c>
       <c r="E14" s="132"/>
-      <c r="F14" s="130">
+      <c r="F14" s="162"/>
+      <c r="G14" s="130">
         <v>11718</v>
       </c>
-      <c r="G14" s="131">
+      <c r="H14" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="106"/>
-    </row>
-    <row r="15" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I14" s="106"/>
+    </row>
+    <row r="15" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A15" s="132">
         <v>69</v>
       </c>
@@ -36214,16 +36355,17 @@
         <v>38143</v>
       </c>
       <c r="E15" s="132"/>
-      <c r="F15" s="130">
+      <c r="F15" s="162"/>
+      <c r="G15" s="130">
         <v>38145</v>
       </c>
-      <c r="G15" s="131">
+      <c r="H15" s="131">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="H15" s="106"/>
-    </row>
-    <row r="16" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I15" s="106"/>
+    </row>
+    <row r="16" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A16" s="132">
         <v>70</v>
       </c>
@@ -36237,16 +36379,17 @@
         <v>35381.199999999997</v>
       </c>
       <c r="E16" s="132"/>
-      <c r="F16" s="130">
+      <c r="F16" s="162"/>
+      <c r="G16" s="130">
         <v>35381.199999999997</v>
       </c>
-      <c r="G16" s="131">
+      <c r="H16" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="106"/>
-    </row>
-    <row r="17" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I16" s="106"/>
+    </row>
+    <row r="17" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A17" s="132">
         <v>71</v>
       </c>
@@ -36260,16 +36403,17 @@
         <v>179707</v>
       </c>
       <c r="E17" s="132"/>
-      <c r="F17" s="130">
+      <c r="F17" s="162"/>
+      <c r="G17" s="130">
         <v>179707</v>
       </c>
-      <c r="G17" s="131">
+      <c r="H17" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H17" s="106"/>
-    </row>
-    <row r="18" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I17" s="106"/>
+    </row>
+    <row r="18" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A18" s="132">
         <v>72</v>
       </c>
@@ -36283,16 +36427,17 @@
         <v>103115.8</v>
       </c>
       <c r="E18" s="132"/>
-      <c r="F18" s="130">
+      <c r="F18" s="162"/>
+      <c r="G18" s="130">
         <v>103121.8</v>
       </c>
-      <c r="G18" s="131">
+      <c r="H18" s="131">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="H18" s="106"/>
-    </row>
-    <row r="19" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I18" s="106"/>
+    </row>
+    <row r="19" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A19" s="132">
         <v>73</v>
       </c>
@@ -36306,16 +36451,17 @@
         <v>18870</v>
       </c>
       <c r="E19" s="132"/>
-      <c r="F19" s="130">
+      <c r="F19" s="162"/>
+      <c r="G19" s="130">
         <v>18870</v>
       </c>
-      <c r="G19" s="131">
+      <c r="H19" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H19" s="106"/>
-    </row>
-    <row r="20" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I19" s="106"/>
+    </row>
+    <row r="20" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A20" s="132">
         <v>74</v>
       </c>
@@ -36329,16 +36475,17 @@
         <v>72558.399999999994</v>
       </c>
       <c r="E20" s="132"/>
-      <c r="F20" s="130">
+      <c r="F20" s="162"/>
+      <c r="G20" s="130">
         <v>72558.399999999994</v>
       </c>
-      <c r="G20" s="131">
+      <c r="H20" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="106"/>
-    </row>
-    <row r="21" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I20" s="106"/>
+    </row>
+    <row r="21" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A21" s="132">
         <v>75</v>
       </c>
@@ -36352,16 +36499,17 @@
         <v>12607</v>
       </c>
       <c r="E21" s="132"/>
-      <c r="F21" s="130">
+      <c r="F21" s="162"/>
+      <c r="G21" s="130">
         <v>12608</v>
       </c>
-      <c r="G21" s="131">
+      <c r="H21" s="131">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="106"/>
-    </row>
-    <row r="22" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I21" s="106"/>
+    </row>
+    <row r="22" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A22" s="132">
         <v>82</v>
       </c>
@@ -36373,16 +36521,17 @@
         <v>0</v>
       </c>
       <c r="E22" s="132"/>
-      <c r="F22" s="130">
+      <c r="F22" s="162"/>
+      <c r="G22" s="130">
         <v>274.60000000000002</v>
       </c>
-      <c r="G22" s="131">
+      <c r="H22" s="131">
         <f t="shared" si="0"/>
         <v>274.60000000000002</v>
       </c>
-      <c r="H22" s="106"/>
-    </row>
-    <row r="23" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I22" s="106"/>
+    </row>
+    <row r="23" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A23" s="132">
         <v>87</v>
       </c>
@@ -36396,16 +36545,17 @@
         <v>30522</v>
       </c>
       <c r="E23" s="132"/>
-      <c r="F23" s="130">
+      <c r="F23" s="162"/>
+      <c r="G23" s="130">
         <v>30522</v>
       </c>
-      <c r="G23" s="131">
+      <c r="H23" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H23" s="106"/>
-    </row>
-    <row r="24" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I23" s="106"/>
+    </row>
+    <row r="24" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A24" s="132">
         <v>88</v>
       </c>
@@ -36419,16 +36569,17 @@
         <v>42174</v>
       </c>
       <c r="E24" s="132"/>
-      <c r="F24" s="130">
+      <c r="F24" s="162"/>
+      <c r="G24" s="130">
         <v>42174</v>
       </c>
-      <c r="G24" s="131">
+      <c r="H24" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="106"/>
-    </row>
-    <row r="25" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I24" s="106"/>
+    </row>
+    <row r="25" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A25" s="132">
         <v>89</v>
       </c>
@@ -36442,16 +36593,17 @@
         <v>0</v>
       </c>
       <c r="E25" s="132"/>
-      <c r="F25" s="130">
+      <c r="F25" s="162"/>
+      <c r="G25" s="130">
         <v>101.9</v>
       </c>
-      <c r="G25" s="131">
+      <c r="H25" s="131">
         <f t="shared" si="0"/>
         <v>101.9</v>
       </c>
-      <c r="H25" s="106"/>
-    </row>
-    <row r="26" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I25" s="106"/>
+    </row>
+    <row r="26" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A26" s="132">
         <v>90</v>
       </c>
@@ -36465,16 +36617,17 @@
         <v>0</v>
       </c>
       <c r="E26" s="132"/>
-      <c r="F26" s="130">
+      <c r="F26" s="162"/>
+      <c r="G26" s="130">
         <v>47842.5</v>
       </c>
-      <c r="G26" s="131">
+      <c r="H26" s="131">
         <f t="shared" si="0"/>
         <v>47842.5</v>
       </c>
-      <c r="H26" s="106"/>
-    </row>
-    <row r="27" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I26" s="106"/>
+    </row>
+    <row r="27" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A27" s="132">
         <v>91</v>
       </c>
@@ -36488,16 +36641,17 @@
         <v>0</v>
       </c>
       <c r="E27" s="132"/>
-      <c r="F27" s="130">
+      <c r="F27" s="162"/>
+      <c r="G27" s="130">
         <v>54.7</v>
       </c>
-      <c r="G27" s="131">
+      <c r="H27" s="131">
         <f t="shared" si="0"/>
         <v>54.7</v>
       </c>
-      <c r="H27" s="106"/>
-    </row>
-    <row r="28" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I27" s="106"/>
+    </row>
+    <row r="28" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A28" s="132">
         <v>92</v>
       </c>
@@ -36511,16 +36665,17 @@
         <v>55276.2</v>
       </c>
       <c r="E28" s="132"/>
-      <c r="F28" s="130">
+      <c r="F28" s="162"/>
+      <c r="G28" s="130">
         <v>55295.6</v>
       </c>
-      <c r="G28" s="131">
+      <c r="H28" s="131">
         <f t="shared" si="0"/>
         <v>19.400000000001455</v>
       </c>
-      <c r="H28" s="106"/>
-    </row>
-    <row r="29" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I28" s="106"/>
+    </row>
+    <row r="29" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A29" s="130">
         <v>93</v>
       </c>
@@ -36534,16 +36689,17 @@
         <v>1076.4000000000001</v>
       </c>
       <c r="E29" s="130"/>
-      <c r="F29" s="130">
+      <c r="F29" s="162"/>
+      <c r="G29" s="130">
         <v>1234.5</v>
       </c>
-      <c r="G29" s="131">
+      <c r="H29" s="131">
         <f t="shared" si="0"/>
         <v>158.09999999999991</v>
       </c>
-      <c r="H29" s="106"/>
-    </row>
-    <row r="30" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I29" s="106"/>
+    </row>
+    <row r="30" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A30" s="132">
         <v>94</v>
       </c>
@@ -36557,16 +36713,17 @@
         <v>26813.1</v>
       </c>
       <c r="E30" s="132"/>
-      <c r="F30" s="130">
+      <c r="F30" s="162"/>
+      <c r="G30" s="130">
         <v>26832.799999999999</v>
       </c>
-      <c r="G30" s="131">
+      <c r="H30" s="131">
         <f t="shared" si="0"/>
         <v>19.700000000000728</v>
       </c>
-      <c r="H30" s="106"/>
-    </row>
-    <row r="31" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I30" s="106"/>
+    </row>
+    <row r="31" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A31" s="130">
         <v>95</v>
       </c>
@@ -36580,16 +36737,17 @@
         <v>26313</v>
       </c>
       <c r="E31" s="130"/>
-      <c r="F31" s="130">
+      <c r="F31" s="162"/>
+      <c r="G31" s="130">
         <v>139657</v>
       </c>
-      <c r="G31" s="131">
+      <c r="H31" s="131">
         <f t="shared" si="0"/>
         <v>113344</v>
       </c>
-      <c r="H31" s="106"/>
-    </row>
-    <row r="32" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I31" s="106"/>
+    </row>
+    <row r="32" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A32" s="132">
         <v>96</v>
       </c>
@@ -36603,16 +36761,17 @@
         <v>16956.2</v>
       </c>
       <c r="E32" s="132"/>
-      <c r="F32" s="130">
+      <c r="F32" s="162"/>
+      <c r="G32" s="130">
         <v>16978.099999999999</v>
       </c>
-      <c r="G32" s="131">
+      <c r="H32" s="131">
         <f t="shared" si="0"/>
         <v>21.899999999997817</v>
       </c>
-      <c r="H32" s="106"/>
-    </row>
-    <row r="33" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I32" s="106"/>
+    </row>
+    <row r="33" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A33" s="130">
         <v>97</v>
       </c>
@@ -36626,16 +36785,17 @@
         <v>36948.800000000003</v>
       </c>
       <c r="E33" s="130"/>
-      <c r="F33" s="130">
+      <c r="F33" s="162"/>
+      <c r="G33" s="130">
         <v>36948.800000000003</v>
       </c>
-      <c r="G33" s="131">
+      <c r="H33" s="131">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H33" s="106"/>
-    </row>
-    <row r="34" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I33" s="106"/>
+    </row>
+    <row r="34" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A34" s="132">
         <v>98</v>
       </c>
@@ -36649,16 +36809,17 @@
         <v>43330.5</v>
       </c>
       <c r="E34" s="132"/>
-      <c r="F34" s="130">
+      <c r="F34" s="162"/>
+      <c r="G34" s="130">
         <v>43364.7</v>
       </c>
-      <c r="G34" s="131">
+      <c r="H34" s="131">
         <f t="shared" si="0"/>
         <v>34.19999999999709</v>
       </c>
-      <c r="H34" s="106"/>
-    </row>
-    <row r="35" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I34" s="106"/>
+    </row>
+    <row r="35" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A35" s="130">
         <v>99</v>
       </c>
@@ -36672,16 +36833,17 @@
         <v>21735.7</v>
       </c>
       <c r="E35" s="130"/>
-      <c r="F35" s="130">
+      <c r="F35" s="162"/>
+      <c r="G35" s="130">
         <v>21789.1</v>
       </c>
-      <c r="G35" s="131">
-        <f t="shared" ref="G35:G54" si="1">F35-D35</f>
+      <c r="H35" s="131">
+        <f t="shared" ref="H35:H54" si="1">G35-D35</f>
         <v>53.399999999997817</v>
       </c>
-      <c r="H35" s="106"/>
-    </row>
-    <row r="36" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I35" s="106"/>
+    </row>
+    <row r="36" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A36" s="132">
         <v>100</v>
       </c>
@@ -36695,16 +36857,17 @@
         <v>28815.3</v>
       </c>
       <c r="E36" s="132"/>
-      <c r="F36" s="130">
+      <c r="F36" s="162"/>
+      <c r="G36" s="130">
         <v>28847.1</v>
       </c>
-      <c r="G36" s="131">
+      <c r="H36" s="131">
         <f t="shared" si="1"/>
         <v>31.799999999999272</v>
       </c>
-      <c r="H36" s="106"/>
-    </row>
-    <row r="37" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I36" s="106"/>
+    </row>
+    <row r="37" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A37" s="130">
         <v>101</v>
       </c>
@@ -36718,16 +36881,17 @@
         <v>30210.7</v>
       </c>
       <c r="E37" s="130"/>
-      <c r="F37" s="130">
+      <c r="F37" s="162"/>
+      <c r="G37" s="130">
         <v>30259.5</v>
       </c>
-      <c r="G37" s="131">
+      <c r="H37" s="131">
         <f t="shared" si="1"/>
         <v>48.799999999999272</v>
       </c>
-      <c r="H37" s="106"/>
-    </row>
-    <row r="38" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I37" s="106"/>
+    </row>
+    <row r="38" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A38" s="132">
         <v>102</v>
       </c>
@@ -36741,16 +36905,17 @@
         <v>1849.3</v>
       </c>
       <c r="E38" s="132"/>
-      <c r="F38" s="130">
+      <c r="F38" s="162"/>
+      <c r="G38" s="130">
         <v>1881.8</v>
       </c>
-      <c r="G38" s="131">
+      <c r="H38" s="131">
         <f t="shared" si="1"/>
         <v>32.5</v>
       </c>
-      <c r="H38" s="106"/>
-    </row>
-    <row r="39" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I38" s="106"/>
+    </row>
+    <row r="39" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A39" s="130">
         <v>103</v>
       </c>
@@ -36764,16 +36929,17 @@
         <v>82275</v>
       </c>
       <c r="E39" s="130"/>
-      <c r="F39" s="130">
+      <c r="F39" s="162"/>
+      <c r="G39" s="130">
         <v>82330</v>
       </c>
-      <c r="G39" s="131">
+      <c r="H39" s="131">
         <f t="shared" si="1"/>
         <v>55</v>
       </c>
-      <c r="H39" s="106"/>
-    </row>
-    <row r="40" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I39" s="106"/>
+    </row>
+    <row r="40" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A40" s="130">
         <v>105</v>
       </c>
@@ -36787,16 +36953,17 @@
         <v>28976.3</v>
       </c>
       <c r="E40" s="130"/>
-      <c r="F40" s="130">
+      <c r="F40" s="162"/>
+      <c r="G40" s="130">
         <v>29012.7</v>
       </c>
-      <c r="G40" s="131">
+      <c r="H40" s="131">
         <f t="shared" si="1"/>
         <v>36.400000000001455</v>
       </c>
-      <c r="H40" s="106"/>
-    </row>
-    <row r="41" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I40" s="106"/>
+    </row>
+    <row r="41" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A41" s="130">
         <v>107</v>
       </c>
@@ -36810,16 +36977,17 @@
         <v>19376</v>
       </c>
       <c r="E41" s="130"/>
-      <c r="F41" s="130"/>
-      <c r="G41" s="131">
+      <c r="F41" s="162"/>
+      <c r="G41" s="130"/>
+      <c r="H41" s="131">
         <f t="shared" si="1"/>
         <v>-19376</v>
       </c>
-      <c r="H41" s="106" t="s">
+      <c r="I41" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="42" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A42" s="130">
         <v>109</v>
       </c>
@@ -36833,18 +37001,19 @@
         <v>29281.599999999999</v>
       </c>
       <c r="E42" s="130"/>
-      <c r="F42" s="130">
+      <c r="F42" s="162"/>
+      <c r="G42" s="130">
         <v>29406.1</v>
       </c>
-      <c r="G42" s="131">
+      <c r="H42" s="131">
         <f t="shared" si="1"/>
         <v>124.5</v>
       </c>
-      <c r="H42" s="106" t="s">
+      <c r="I42" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="43" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A43" s="130">
         <v>111</v>
       </c>
@@ -36858,18 +37027,19 @@
         <v>5509</v>
       </c>
       <c r="E43" s="130"/>
-      <c r="F43" s="130">
+      <c r="F43" s="162"/>
+      <c r="G43" s="130">
         <v>5516</v>
       </c>
-      <c r="G43" s="131">
+      <c r="H43" s="131">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="H43" s="106" t="s">
+      <c r="I43" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="44" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A44" s="130">
         <v>113</v>
       </c>
@@ -36883,18 +37053,19 @@
         <v>38016.9</v>
       </c>
       <c r="E44" s="130"/>
-      <c r="F44" s="130">
+      <c r="F44" s="162"/>
+      <c r="G44" s="130">
         <v>38086</v>
       </c>
-      <c r="G44" s="131">
+      <c r="H44" s="131">
         <f t="shared" si="1"/>
         <v>69.099999999998545</v>
       </c>
-      <c r="H44" s="106" t="s">
+      <c r="I44" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="45" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A45" s="130">
         <v>115</v>
       </c>
@@ -36908,18 +37079,19 @@
         <v>71144.2</v>
       </c>
       <c r="E45" s="130"/>
-      <c r="F45" s="130">
+      <c r="F45" s="162"/>
+      <c r="G45" s="130">
         <v>71214.8</v>
       </c>
-      <c r="G45" s="131">
+      <c r="H45" s="131">
         <f t="shared" si="1"/>
         <v>70.600000000005821</v>
       </c>
-      <c r="H45" s="106" t="s">
+      <c r="I45" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="46" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A46" s="130">
         <v>117</v>
       </c>
@@ -36933,18 +37105,19 @@
         <v>63803.5</v>
       </c>
       <c r="E46" s="130"/>
-      <c r="F46" s="130">
+      <c r="F46" s="162"/>
+      <c r="G46" s="130">
         <v>63860.4</v>
       </c>
-      <c r="G46" s="131">
+      <c r="H46" s="131">
         <f t="shared" si="1"/>
         <v>56.900000000001455</v>
       </c>
-      <c r="H46" s="106" t="s">
+      <c r="I46" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="47" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A47" s="130">
         <v>119</v>
       </c>
@@ -36958,18 +37131,19 @@
         <v>29124.2</v>
       </c>
       <c r="E47" s="130"/>
-      <c r="F47" s="130">
+      <c r="F47" s="162"/>
+      <c r="G47" s="130">
         <v>29208.6</v>
       </c>
-      <c r="G47" s="131">
+      <c r="H47" s="131">
         <f t="shared" si="1"/>
         <v>84.399999999997817</v>
       </c>
-      <c r="H47" s="106" t="s">
+      <c r="I47" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="48" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A48" s="130">
         <v>121</v>
       </c>
@@ -36983,18 +37157,19 @@
         <v>9600.1</v>
       </c>
       <c r="E48" s="130"/>
-      <c r="F48" s="130">
+      <c r="F48" s="162"/>
+      <c r="G48" s="130">
         <v>9668.1</v>
       </c>
-      <c r="G48" s="131">
+      <c r="H48" s="131">
         <f t="shared" si="1"/>
         <v>68</v>
       </c>
-      <c r="H48" s="106" t="s">
+      <c r="I48" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="49" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A49" s="130">
         <v>123</v>
       </c>
@@ -37008,18 +37183,19 @@
         <v>89289.8</v>
       </c>
       <c r="E49" s="130"/>
-      <c r="F49" s="130">
+      <c r="F49" s="162"/>
+      <c r="G49" s="130">
         <v>89352.7</v>
       </c>
-      <c r="G49" s="131">
+      <c r="H49" s="131">
         <f t="shared" si="1"/>
         <v>62.899999999994179</v>
       </c>
-      <c r="H49" s="106" t="s">
+      <c r="I49" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="50" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A50" s="130">
         <v>125</v>
       </c>
@@ -37033,18 +37209,19 @@
         <v>89182.7</v>
       </c>
       <c r="E50" s="130"/>
-      <c r="F50" s="130">
+      <c r="F50" s="162"/>
+      <c r="G50" s="130">
         <v>89225.2</v>
       </c>
-      <c r="G50" s="131">
+      <c r="H50" s="131">
         <f t="shared" si="1"/>
         <v>42.5</v>
       </c>
-      <c r="H50" s="106" t="s">
+      <c r="I50" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="51" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A51" s="130">
         <v>127</v>
       </c>
@@ -37058,18 +37235,19 @@
         <v>25290.799999999999</v>
       </c>
       <c r="E51" s="130"/>
-      <c r="F51" s="130">
+      <c r="F51" s="162"/>
+      <c r="G51" s="130">
         <v>25372.1</v>
       </c>
-      <c r="G51" s="131">
+      <c r="H51" s="131">
         <f t="shared" si="1"/>
         <v>81.299999999999272</v>
       </c>
-      <c r="H51" s="106" t="s">
+      <c r="I51" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="52" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A52" s="130">
         <v>163</v>
       </c>
@@ -37083,14 +37261,15 @@
         <v>35892.800000000003</v>
       </c>
       <c r="E52" s="130"/>
-      <c r="F52" s="130"/>
-      <c r="G52" s="131">
+      <c r="F52" s="162"/>
+      <c r="G52" s="130"/>
+      <c r="H52" s="131">
         <f t="shared" si="1"/>
         <v>-35892.800000000003</v>
       </c>
-      <c r="H52" s="106"/>
-    </row>
-    <row r="53" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+      <c r="I52" s="106"/>
+    </row>
+    <row r="53" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A53" s="130">
         <v>186</v>
       </c>
@@ -37102,18 +37281,19 @@
         <v>0</v>
       </c>
       <c r="E53" s="130"/>
-      <c r="F53" s="130">
+      <c r="F53" s="162"/>
+      <c r="G53" s="130">
         <v>488.5</v>
       </c>
-      <c r="G53" s="131">
+      <c r="H53" s="131">
         <f t="shared" si="1"/>
         <v>488.5</v>
       </c>
-      <c r="H53" s="106" t="s">
+      <c r="I53" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="23.25" x14ac:dyDescent="0.7">
+    <row r="54" spans="1:9" ht="23.25" x14ac:dyDescent="0.7">
       <c r="A54" s="130">
         <v>179</v>
       </c>
@@ -37125,23 +37305,24 @@
         <v>0</v>
       </c>
       <c r="E54" s="133"/>
-      <c r="F54" s="130">
+      <c r="F54" s="162"/>
+      <c r="G54" s="130">
         <v>649.9</v>
       </c>
-      <c r="G54" s="131">
+      <c r="H54" s="131">
         <f t="shared" si="1"/>
         <v>649.9</v>
       </c>
-      <c r="H54" s="106" t="s">
+      <c r="I54" s="106" t="s">
         <v>1183</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G52">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H52">
     <sortCondition ref="A2:A52"/>
   </sortState>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1:H1048576 E1:E1048576" xr:uid="{2C5E24F2-5EB5-480F-A2A4-FF792E3FE22F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1:I1048576 E1:E1048576 F55:F1048576" xr:uid="{2C5E24F2-5EB5-480F-A2A4-FF792E3FE22F}">
       <formula1>"Yes"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
NEw elec and water meters installed
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2597" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6260444-4B2A-403D-B895-B1128DEFD2DC}"/>
+  <xr:revisionPtr revIDLastSave="2644" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{671B272E-058D-41BA-9C16-F8B3AC8C9731}"/>
   <bookViews>
     <workbookView xWindow="43080" yWindow="-7455" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5006" uniqueCount="1197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5019" uniqueCount="1203">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -3638,6 +3638,24 @@
   </si>
   <si>
     <t>10192063</t>
+  </si>
+  <si>
+    <t>Kamstrup</t>
+  </si>
+  <si>
+    <t>FlowIQ2200</t>
+  </si>
+  <si>
+    <t>54554431</t>
+  </si>
+  <si>
+    <t>10192057</t>
+  </si>
+  <si>
+    <t>10192056</t>
+  </si>
+  <si>
+    <t>10191967</t>
   </si>
 </sst>
 </file>
@@ -5335,7 +5353,9 @@
       <c r="B2" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="2"/>
+      <c r="C2" s="2">
+        <v>14558066321</v>
+      </c>
       <c r="D2" s="2">
         <v>82929702</v>
       </c>
@@ -5348,14 +5368,18 @@
       <c r="G2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="7" t="s">
+        <v>64</v>
+      </c>
       <c r="I2" s="39" t="s">
         <v>22</v>
       </c>
       <c r="J2" s="9">
         <v>0</v>
       </c>
-      <c r="K2" s="2"/>
+      <c r="K2" s="4">
+        <v>46219</v>
+      </c>
       <c r="L2" s="11" t="b">
         <v>0</v>
       </c>
@@ -5383,7 +5407,9 @@
       <c r="B3" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="2"/>
+      <c r="C3" s="2">
+        <v>14558069515</v>
+      </c>
       <c r="D3" s="2">
         <v>82929702</v>
       </c>
@@ -5396,14 +5422,18 @@
       <c r="G3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="2"/>
+      <c r="H3" s="7" t="s">
+        <v>64</v>
+      </c>
       <c r="I3" s="39" t="s">
         <v>22</v>
       </c>
       <c r="J3" s="9">
         <v>0</v>
       </c>
-      <c r="K3" s="2"/>
+      <c r="K3" s="4">
+        <v>46219</v>
+      </c>
       <c r="L3" s="11" t="b">
         <v>0</v>
       </c>
@@ -5431,7 +5461,9 @@
       <c r="B4" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="2"/>
+      <c r="C4" s="2">
+        <v>14558069051</v>
+      </c>
       <c r="D4" s="2">
         <v>82929702</v>
       </c>
@@ -5444,14 +5476,18 @@
       <c r="G4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="I4" s="39" t="s">
         <v>22</v>
       </c>
       <c r="J4" s="9">
         <v>0</v>
       </c>
-      <c r="K4" s="2"/>
+      <c r="K4" s="4">
+        <v>46219</v>
+      </c>
       <c r="L4" s="11" t="b">
         <v>0</v>
       </c>
@@ -5479,7 +5515,9 @@
       <c r="B5" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="2"/>
+      <c r="C5" s="2">
+        <v>14558069440</v>
+      </c>
       <c r="D5" s="2">
         <v>82929702</v>
       </c>
@@ -5492,14 +5530,18 @@
       <c r="G5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="2"/>
+      <c r="H5" s="7" t="s">
+        <v>64</v>
+      </c>
       <c r="I5" s="39" t="s">
         <v>22</v>
       </c>
       <c r="J5" s="9">
         <v>0</v>
       </c>
-      <c r="K5" s="2"/>
+      <c r="K5" s="4">
+        <v>46219</v>
+      </c>
       <c r="L5" s="11" t="b">
         <v>0</v>
       </c>
@@ -5527,7 +5569,9 @@
       <c r="B6" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="2"/>
+      <c r="C6" s="2">
+        <v>14558068418</v>
+      </c>
       <c r="D6" s="2">
         <v>82929702</v>
       </c>
@@ -5540,14 +5584,18 @@
       <c r="G6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H6" s="2"/>
+      <c r="H6" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="I6" s="39" t="s">
         <v>22</v>
       </c>
       <c r="J6" s="9">
         <v>0</v>
       </c>
-      <c r="K6" s="2"/>
+      <c r="K6" s="4">
+        <v>46219</v>
+      </c>
       <c r="L6" s="11" t="b">
         <v>0</v>
       </c>
@@ -5575,7 +5623,9 @@
       <c r="B7" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="2">
+        <v>14558068459</v>
+      </c>
       <c r="D7" s="2">
         <v>82929702</v>
       </c>
@@ -5588,14 +5638,18 @@
       <c r="G7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="2"/>
+      <c r="H7" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="I7" s="39" t="s">
         <v>22</v>
       </c>
       <c r="J7" s="9">
         <v>0</v>
       </c>
-      <c r="K7" s="2"/>
+      <c r="K7" s="4">
+        <v>46219</v>
+      </c>
       <c r="L7" s="11" t="b">
         <v>0</v>
       </c>
@@ -5623,7 +5677,9 @@
       <c r="B8" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="2">
+        <v>14558069572</v>
+      </c>
       <c r="D8" s="2">
         <v>82929702</v>
       </c>
@@ -5636,14 +5692,18 @@
       <c r="G8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="I8" s="39" t="s">
         <v>22</v>
       </c>
       <c r="J8" s="9">
         <v>0</v>
       </c>
-      <c r="K8" s="2"/>
+      <c r="K8" s="4">
+        <v>46219</v>
+      </c>
       <c r="L8" s="11" t="b">
         <v>0</v>
       </c>
@@ -5671,7 +5731,9 @@
       <c r="B9" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="2">
+        <v>14558069408</v>
+      </c>
       <c r="D9" s="2">
         <v>82929702</v>
       </c>
@@ -5684,14 +5746,18 @@
       <c r="G9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H9" s="2"/>
+      <c r="H9" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="I9" s="39" t="s">
         <v>22</v>
       </c>
       <c r="J9" s="9">
         <v>0</v>
       </c>
-      <c r="K9" s="2"/>
+      <c r="K9" s="4">
+        <v>46219</v>
+      </c>
       <c r="L9" s="11" t="b">
         <v>0</v>
       </c>
@@ -5719,7 +5785,9 @@
       <c r="B10" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="2"/>
+      <c r="C10" s="2">
+        <v>14558069523</v>
+      </c>
       <c r="D10" s="2">
         <v>82929702</v>
       </c>
@@ -5732,14 +5800,18 @@
       <c r="G10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H10" s="2"/>
+      <c r="H10" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="I10" s="39" t="s">
         <v>22</v>
       </c>
       <c r="J10" s="9">
         <v>0</v>
       </c>
-      <c r="K10" s="2"/>
+      <c r="K10" s="4">
+        <v>46219</v>
+      </c>
       <c r="L10" s="11" t="b">
         <v>0</v>
       </c>
@@ -23887,7 +23959,9 @@
       <c r="B175" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="C175" s="53"/>
+      <c r="C175" s="53" t="s">
+        <v>1202</v>
+      </c>
       <c r="D175" s="53" t="s">
         <v>283</v>
       </c>
@@ -23897,10 +23971,14 @@
       <c r="F175" s="53" t="s">
         <v>285</v>
       </c>
-      <c r="G175" s="3"/>
-      <c r="H175" s="3"/>
+      <c r="G175" s="3">
+        <v>6.7000000000000004E-2</v>
+      </c>
+      <c r="H175" s="57">
+        <v>46219</v>
+      </c>
       <c r="I175" s="21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J175" s="63" t="s">
         <v>244</v>
@@ -23932,18 +24010,24 @@
       <c r="B176" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="C176" s="53"/>
+      <c r="C176" s="53" t="s">
+        <v>1199</v>
+      </c>
       <c r="D176" s="53" t="s">
-        <v>283</v>
+        <v>1197</v>
       </c>
       <c r="E176" s="53" t="s">
-        <v>284</v>
+        <v>1198</v>
       </c>
       <c r="F176" s="53" t="s">
         <v>285</v>
       </c>
-      <c r="G176" s="3"/>
-      <c r="H176" s="3"/>
+      <c r="G176" s="3">
+        <v>0.161</v>
+      </c>
+      <c r="H176" s="57">
+        <v>46219</v>
+      </c>
       <c r="I176" s="21" t="b">
         <v>0</v>
       </c>
@@ -24028,7 +24112,9 @@
       <c r="B178" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="C178" s="53"/>
+      <c r="C178" s="53" t="s">
+        <v>1200</v>
+      </c>
       <c r="D178" s="53" t="s">
         <v>283</v>
       </c>
@@ -24038,10 +24124,14 @@
       <c r="F178" s="53" t="s">
         <v>285</v>
       </c>
-      <c r="G178" s="3"/>
-      <c r="H178" s="3"/>
+      <c r="G178" s="3">
+        <v>9.1999999999999998E-2</v>
+      </c>
+      <c r="H178" s="57">
+        <v>46219</v>
+      </c>
       <c r="I178" s="21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J178" s="63" t="s">
         <v>250</v>
@@ -24073,7 +24163,9 @@
       <c r="B179" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="C179" s="53"/>
+      <c r="C179" s="53" t="s">
+        <v>1201</v>
+      </c>
       <c r="D179" s="53" t="s">
         <v>283</v>
       </c>
@@ -24083,10 +24175,14 @@
       <c r="F179" s="53" t="s">
         <v>285</v>
       </c>
-      <c r="G179" s="3"/>
-      <c r="H179" s="3"/>
+      <c r="G179" s="3">
+        <v>0.09</v>
+      </c>
+      <c r="H179" s="57">
+        <v>46219</v>
+      </c>
       <c r="I179" s="21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J179" s="63" t="s">
         <v>250</v>

</xml_diff>

<commit_message>
NEw elec meters istalled
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2745" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD9F566C-F058-4A88-B16A-1AEEDA2C67FB}"/>
+  <xr:revisionPtr revIDLastSave="2772" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62980A75-8457-4502-B976-4FDC60B88EDD}"/>
   <bookViews>
     <workbookView xWindow="43080" yWindow="-7455" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,6 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'FS Water'!$A$1:$Q$193</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5036" uniqueCount="1204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5044" uniqueCount="1204">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -4761,14 +4762,14 @@
     <xf numFmtId="14" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -6556,7 +6557,7 @@
       <c r="B24" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="161">
+      <c r="C24" s="159">
         <v>14558068921</v>
       </c>
       <c r="D24" s="2">
@@ -9768,7 +9769,7 @@
       <c r="B83" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="C83" s="161">
+      <c r="C83" s="159">
         <v>14558069077</v>
       </c>
       <c r="D83" s="2">
@@ -13232,7 +13233,9 @@
       <c r="B147" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C147" s="2"/>
+      <c r="C147" s="2">
+        <v>14558069812</v>
+      </c>
       <c r="D147" s="2">
         <v>71205556</v>
       </c>
@@ -13245,14 +13248,18 @@
       <c r="G147" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H147" s="2"/>
+      <c r="H147" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="I147" s="31" t="s">
         <v>46</v>
       </c>
       <c r="J147" s="9">
         <v>0</v>
       </c>
-      <c r="K147" s="2"/>
+      <c r="K147" s="4">
+        <v>46224</v>
+      </c>
       <c r="L147" s="11" t="b">
         <v>0</v>
       </c>
@@ -13328,7 +13335,9 @@
       <c r="B149" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C149" s="2"/>
+      <c r="C149" s="2">
+        <v>14558069754</v>
+      </c>
       <c r="D149" s="2">
         <v>71205556</v>
       </c>
@@ -13341,14 +13350,18 @@
       <c r="G149" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H149" s="2"/>
+      <c r="H149" s="8" t="s">
+        <v>33</v>
+      </c>
       <c r="I149" s="31" t="s">
         <v>46</v>
       </c>
       <c r="J149" s="9">
         <v>0</v>
       </c>
-      <c r="K149" s="2"/>
+      <c r="K149" s="4">
+        <v>46224</v>
+      </c>
       <c r="L149" s="11" t="b">
         <v>0</v>
       </c>
@@ -13376,7 +13389,9 @@
       <c r="B150" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C150" s="2"/>
+      <c r="C150" s="2">
+        <v>14558067931</v>
+      </c>
       <c r="D150" s="2">
         <v>71205556</v>
       </c>
@@ -13389,14 +13404,18 @@
       <c r="G150" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H150" s="2"/>
+      <c r="H150" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="I150" s="31" t="s">
         <v>46</v>
       </c>
       <c r="J150" s="9">
         <v>0</v>
       </c>
-      <c r="K150" s="2"/>
+      <c r="K150" s="4">
+        <v>46224</v>
+      </c>
       <c r="L150" s="11" t="b">
         <v>0</v>
       </c>
@@ -13424,7 +13443,9 @@
       <c r="B151" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C151" s="2"/>
+      <c r="C151" s="2">
+        <v>14558069788</v>
+      </c>
       <c r="D151" s="2">
         <v>71205556</v>
       </c>
@@ -13437,14 +13458,18 @@
       <c r="G151" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H151" s="2"/>
+      <c r="H151" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="I151" s="31" t="s">
         <v>46</v>
       </c>
       <c r="J151" s="9">
         <v>0</v>
       </c>
-      <c r="K151" s="2"/>
+      <c r="K151" s="4">
+        <v>46224</v>
+      </c>
       <c r="L151" s="11" t="b">
         <v>0</v>
       </c>
@@ -13472,7 +13497,9 @@
       <c r="B152" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C152" s="2"/>
+      <c r="C152" s="2">
+        <v>14558067956</v>
+      </c>
       <c r="D152" s="2">
         <v>71205556</v>
       </c>
@@ -13485,14 +13512,18 @@
       <c r="G152" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H152" s="2"/>
+      <c r="H152" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="I152" s="31" t="s">
         <v>46</v>
       </c>
       <c r="J152" s="9">
         <v>0</v>
       </c>
-      <c r="K152" s="2"/>
+      <c r="K152" s="4">
+        <v>46224</v>
+      </c>
       <c r="L152" s="11" t="b">
         <v>0</v>
       </c>
@@ -13520,7 +13551,9 @@
       <c r="B153" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C153" s="2"/>
+      <c r="C153" s="2">
+        <v>14558069747</v>
+      </c>
       <c r="D153" s="2">
         <v>71205556</v>
       </c>
@@ -13533,14 +13566,18 @@
       <c r="G153" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H153" s="2"/>
+      <c r="H153" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="I153" s="31" t="s">
         <v>46</v>
       </c>
       <c r="J153" s="9">
         <v>0</v>
       </c>
-      <c r="K153" s="2"/>
+      <c r="K153" s="4">
+        <v>46224</v>
+      </c>
       <c r="L153" s="11" t="b">
         <v>0</v>
       </c>
@@ -13568,7 +13605,9 @@
       <c r="B154" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C154" s="2"/>
+      <c r="C154" s="2">
+        <v>14558069879</v>
+      </c>
       <c r="D154" s="2">
         <v>71205556</v>
       </c>
@@ -13581,14 +13620,18 @@
       <c r="G154" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H154" s="2"/>
+      <c r="H154" s="8" t="s">
+        <v>33</v>
+      </c>
       <c r="I154" s="31" t="s">
         <v>46</v>
       </c>
       <c r="J154" s="9">
         <v>0</v>
       </c>
-      <c r="K154" s="2"/>
+      <c r="K154" s="4">
+        <v>46224</v>
+      </c>
       <c r="L154" s="11" t="b">
         <v>0</v>
       </c>
@@ -13616,7 +13659,9 @@
       <c r="B155" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C155" s="2"/>
+      <c r="C155" s="2">
+        <v>14558069861</v>
+      </c>
       <c r="D155" s="2">
         <v>71205556</v>
       </c>
@@ -13629,14 +13674,18 @@
       <c r="G155" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H155" s="2"/>
+      <c r="H155" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="I155" s="31" t="s">
         <v>46</v>
       </c>
       <c r="J155" s="9">
         <v>0</v>
       </c>
-      <c r="K155" s="2"/>
+      <c r="K155" s="4">
+        <v>46224</v>
+      </c>
       <c r="L155" s="11" t="b">
         <v>0</v>
       </c>
@@ -15747,12 +15796,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:Q204"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.46484375" customWidth="1"/>
-    <col min="3" max="3" width="30.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.86328125" customWidth="1"/>
     <col min="4" max="4" width="21.59765625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.73046875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25.59765625" bestFit="1" customWidth="1"/>
@@ -15820,7 +15870,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
         <v>116</v>
       </c>
@@ -15865,7 +15915,7 @@
       </c>
       <c r="Q2" s="17"/>
     </row>
-    <row r="3" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="23" t="s">
         <v>119</v>
       </c>
@@ -15910,7 +15960,7 @@
       </c>
       <c r="Q3" s="17"/>
     </row>
-    <row r="4" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
         <v>120</v>
       </c>
@@ -15955,7 +16005,7 @@
       </c>
       <c r="Q4" s="17"/>
     </row>
-    <row r="5" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
         <v>122</v>
       </c>
@@ -16000,7 +16050,7 @@
       </c>
       <c r="Q5" s="17"/>
     </row>
-    <row r="6" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
         <v>123</v>
       </c>
@@ -16045,7 +16095,7 @@
       </c>
       <c r="Q6" s="17"/>
     </row>
-    <row r="7" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
         <v>124</v>
       </c>
@@ -16090,7 +16140,7 @@
       </c>
       <c r="Q7" s="17"/>
     </row>
-    <row r="8" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">
         <v>125</v>
       </c>
@@ -16135,7 +16185,7 @@
       </c>
       <c r="Q8" s="17"/>
     </row>
-    <row r="9" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="23" t="s">
         <v>126</v>
       </c>
@@ -16180,7 +16230,7 @@
       </c>
       <c r="Q9" s="17"/>
     </row>
-    <row r="10" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="23" t="s">
         <v>127</v>
       </c>
@@ -16225,7 +16275,7 @@
       </c>
       <c r="Q10" s="17"/>
     </row>
-    <row r="11" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="23" t="s">
         <v>150</v>
       </c>
@@ -16270,7 +16320,7 @@
       </c>
       <c r="Q11" s="17"/>
     </row>
-    <row r="12" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="23" t="s">
         <v>152</v>
       </c>
@@ -16315,7 +16365,7 @@
       </c>
       <c r="Q12" s="17"/>
     </row>
-    <row r="13" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="23" t="s">
         <v>153</v>
       </c>
@@ -16360,7 +16410,7 @@
       </c>
       <c r="Q13" s="17"/>
     </row>
-    <row r="14" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="23" t="s">
         <v>154</v>
       </c>
@@ -16405,7 +16455,7 @@
       </c>
       <c r="Q14" s="17"/>
     </row>
-    <row r="15" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="23" t="s">
         <v>155</v>
       </c>
@@ -16450,7 +16500,7 @@
       </c>
       <c r="Q15" s="17"/>
     </row>
-    <row r="16" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="23" t="s">
         <v>156</v>
       </c>
@@ -16495,7 +16545,7 @@
       </c>
       <c r="Q16" s="17"/>
     </row>
-    <row r="17" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="23" t="s">
         <v>157</v>
       </c>
@@ -16540,7 +16590,7 @@
       </c>
       <c r="Q17" s="17"/>
     </row>
-    <row r="18" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="23" t="s">
         <v>158</v>
       </c>
@@ -16585,7 +16635,7 @@
       </c>
       <c r="Q18" s="17"/>
     </row>
-    <row r="19" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="23" t="s">
         <v>160</v>
       </c>
@@ -16630,7 +16680,7 @@
       </c>
       <c r="Q19" s="17"/>
     </row>
-    <row r="20" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="23" t="s">
         <v>181</v>
       </c>
@@ -16675,7 +16725,7 @@
       </c>
       <c r="Q20" s="17"/>
     </row>
-    <row r="21" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="23" t="s">
         <v>183</v>
       </c>
@@ -16720,7 +16770,7 @@
       </c>
       <c r="Q21" s="17"/>
     </row>
-    <row r="22" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="23" t="s">
         <v>185</v>
       </c>
@@ -16765,7 +16815,7 @@
       </c>
       <c r="Q22" s="17"/>
     </row>
-    <row r="23" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="23" t="s">
         <v>186</v>
       </c>
@@ -16810,7 +16860,7 @@
       </c>
       <c r="Q23" s="17"/>
     </row>
-    <row r="24" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="23" t="s">
         <v>187</v>
       </c>
@@ -16855,7 +16905,7 @@
       </c>
       <c r="Q24" s="17"/>
     </row>
-    <row r="25" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="23" t="s">
         <v>188</v>
       </c>
@@ -16900,7 +16950,7 @@
       </c>
       <c r="Q25" s="17"/>
     </row>
-    <row r="26" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="23" t="s">
         <v>203</v>
       </c>
@@ -16945,7 +16995,7 @@
       </c>
       <c r="Q26" s="17"/>
     </row>
-    <row r="27" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="23" t="s">
         <v>205</v>
       </c>
@@ -16990,7 +17040,7 @@
       </c>
       <c r="Q27" s="17"/>
     </row>
-    <row r="28" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="23" t="s">
         <v>206</v>
       </c>
@@ -17035,7 +17085,7 @@
       </c>
       <c r="Q28" s="17"/>
     </row>
-    <row r="29" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="23" t="s">
         <v>207</v>
       </c>
@@ -17080,7 +17130,7 @@
       </c>
       <c r="Q29" s="17"/>
     </row>
-    <row r="30" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="23" t="s">
         <v>208</v>
       </c>
@@ -17125,7 +17175,7 @@
       </c>
       <c r="Q30" s="17"/>
     </row>
-    <row r="31" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="23" t="s">
         <v>209</v>
       </c>
@@ -17170,7 +17220,7 @@
       </c>
       <c r="Q31" s="17"/>
     </row>
-    <row r="32" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="23" t="s">
         <v>210</v>
       </c>
@@ -17215,7 +17265,7 @@
       </c>
       <c r="Q32" s="17"/>
     </row>
-    <row r="33" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="23" t="s">
         <v>211</v>
       </c>
@@ -17260,7 +17310,7 @@
       </c>
       <c r="Q33" s="17"/>
     </row>
-    <row r="34" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="23" t="s">
         <v>212</v>
       </c>
@@ -20881,7 +20931,7 @@
         <v>46216</v>
       </c>
     </row>
-    <row r="105" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="23" t="s">
         <v>139</v>
       </c>
@@ -20979,7 +21029,7 @@
         <v>46206</v>
       </c>
     </row>
-    <row r="107" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="23" t="s">
         <v>141</v>
       </c>
@@ -21075,7 +21125,7 @@
       </c>
       <c r="Q108" s="17"/>
     </row>
-    <row r="109" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="23" t="s">
         <v>144</v>
       </c>
@@ -21173,7 +21223,7 @@
         <v>46206</v>
       </c>
     </row>
-    <row r="111" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="23" t="s">
         <v>146</v>
       </c>
@@ -21269,7 +21319,7 @@
       </c>
       <c r="Q112" s="17"/>
     </row>
-    <row r="113" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="23" t="s">
         <v>105</v>
       </c>
@@ -21365,7 +21415,7 @@
       </c>
       <c r="Q114" s="17"/>
     </row>
-    <row r="115" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="23" t="s">
         <v>108</v>
       </c>
@@ -21461,7 +21511,7 @@
       </c>
       <c r="Q116" s="17"/>
     </row>
-    <row r="117" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="23" t="s">
         <v>109</v>
       </c>
@@ -21557,7 +21607,7 @@
       </c>
       <c r="Q118" s="17"/>
     </row>
-    <row r="119" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="23" t="s">
         <v>111</v>
       </c>
@@ -21653,7 +21703,7 @@
       </c>
       <c r="Q120" s="17"/>
     </row>
-    <row r="121" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="23" t="s">
         <v>113</v>
       </c>
@@ -21749,7 +21799,7 @@
       </c>
       <c r="Q122" s="17"/>
     </row>
-    <row r="123" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="23" t="s">
         <v>74</v>
       </c>
@@ -21845,7 +21895,7 @@
       </c>
       <c r="Q124" s="17"/>
     </row>
-    <row r="125" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="23" t="s">
         <v>77</v>
       </c>
@@ -21943,7 +21993,7 @@
         <v>46206</v>
       </c>
     </row>
-    <row r="127" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="23" t="s">
         <v>81</v>
       </c>
@@ -22039,7 +22089,7 @@
       </c>
       <c r="Q128" s="17"/>
     </row>
-    <row r="129" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="23" t="s">
         <v>83</v>
       </c>
@@ -22084,7 +22134,7 @@
       </c>
       <c r="Q129" s="17"/>
     </row>
-    <row r="130" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="23" t="s">
         <v>84</v>
       </c>
@@ -22129,7 +22179,7 @@
       </c>
       <c r="Q130" s="17"/>
     </row>
-    <row r="131" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="23" t="s">
         <v>85</v>
       </c>
@@ -22174,7 +22224,7 @@
       </c>
       <c r="Q131" s="17"/>
     </row>
-    <row r="132" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="23" t="s">
         <v>86</v>
       </c>
@@ -22219,7 +22269,7 @@
       </c>
       <c r="Q132" s="17"/>
     </row>
-    <row r="133" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="23" t="s">
         <v>260</v>
       </c>
@@ -22264,7 +22314,7 @@
       </c>
       <c r="Q133" s="17"/>
     </row>
-    <row r="134" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="23" t="s">
         <v>263</v>
       </c>
@@ -22309,7 +22359,7 @@
       </c>
       <c r="Q134" s="17"/>
     </row>
-    <row r="135" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="23" t="s">
         <v>264</v>
       </c>
@@ -22354,7 +22404,7 @@
       </c>
       <c r="Q135" s="17"/>
     </row>
-    <row r="136" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="23" t="s">
         <v>265</v>
       </c>
@@ -22399,7 +22449,7 @@
       </c>
       <c r="Q136" s="17"/>
     </row>
-    <row r="137" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" s="23" t="s">
         <v>266</v>
       </c>
@@ -22444,7 +22494,7 @@
       </c>
       <c r="Q137" s="17"/>
     </row>
-    <row r="138" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="23" t="s">
         <v>267</v>
       </c>
@@ -22489,7 +22539,7 @@
       </c>
       <c r="Q138" s="17"/>
     </row>
-    <row r="139" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" s="23" t="s">
         <v>268</v>
       </c>
@@ -22534,7 +22584,7 @@
       </c>
       <c r="Q139" s="17"/>
     </row>
-    <row r="140" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" s="23" t="s">
         <v>269</v>
       </c>
@@ -22579,7 +22629,7 @@
       </c>
       <c r="Q140" s="17"/>
     </row>
-    <row r="141" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" s="23" t="s">
         <v>35</v>
       </c>
@@ -22624,7 +22674,7 @@
       </c>
       <c r="Q141" s="17"/>
     </row>
-    <row r="142" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" s="23" t="s">
         <v>38</v>
       </c>
@@ -22669,7 +22719,7 @@
       </c>
       <c r="Q142" s="17"/>
     </row>
-    <row r="143" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" s="23" t="s">
         <v>40</v>
       </c>
@@ -22714,7 +22764,7 @@
       </c>
       <c r="Q143" s="17"/>
     </row>
-    <row r="144" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="23" t="s">
         <v>41</v>
       </c>
@@ -22759,7 +22809,7 @@
       </c>
       <c r="Q144" s="17"/>
     </row>
-    <row r="145" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" s="23" t="s">
         <v>42</v>
       </c>
@@ -22804,7 +22854,7 @@
       </c>
       <c r="Q145" s="17"/>
     </row>
-    <row r="146" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" s="23" t="s">
         <v>43</v>
       </c>
@@ -22849,7 +22899,7 @@
       </c>
       <c r="Q146" s="17"/>
     </row>
-    <row r="147" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="23" t="s">
         <v>45</v>
       </c>
@@ -22894,7 +22944,7 @@
       </c>
       <c r="Q147" s="17"/>
     </row>
-    <row r="148" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="23" t="s">
         <v>44</v>
       </c>
@@ -22939,7 +22989,7 @@
       </c>
       <c r="Q148" s="17"/>
     </row>
-    <row r="149" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="23" t="s">
         <v>47</v>
       </c>
@@ -22984,7 +23034,7 @@
       </c>
       <c r="Q149" s="17"/>
     </row>
-    <row r="150" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" s="23" t="s">
         <v>48</v>
       </c>
@@ -23029,7 +23079,7 @@
       </c>
       <c r="Q150" s="17"/>
     </row>
-    <row r="151" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" s="23" t="s">
         <v>49</v>
       </c>
@@ -23074,7 +23124,7 @@
       </c>
       <c r="Q151" s="17"/>
     </row>
-    <row r="152" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" s="23" t="s">
         <v>50</v>
       </c>
@@ -23119,7 +23169,7 @@
       </c>
       <c r="Q152" s="17"/>
     </row>
-    <row r="153" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" s="23" t="s">
         <v>51</v>
       </c>
@@ -23164,7 +23214,7 @@
       </c>
       <c r="Q153" s="17"/>
     </row>
-    <row r="154" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="23" t="s">
         <v>52</v>
       </c>
@@ -23209,7 +23259,7 @@
       </c>
       <c r="Q154" s="17"/>
     </row>
-    <row r="155" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="23" t="s">
         <v>53</v>
       </c>
@@ -23254,7 +23304,7 @@
       </c>
       <c r="Q155" s="17"/>
     </row>
-    <row r="156" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" s="23" t="s">
         <v>54</v>
       </c>
@@ -23299,7 +23349,7 @@
       </c>
       <c r="Q156" s="17"/>
     </row>
-    <row r="157" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" s="23" t="s">
         <v>57</v>
       </c>
@@ -23344,7 +23394,7 @@
       </c>
       <c r="Q157" s="17"/>
     </row>
-    <row r="158" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" s="23" t="s">
         <v>58</v>
       </c>
@@ -23389,7 +23439,7 @@
       </c>
       <c r="Q158" s="17"/>
     </row>
-    <row r="159" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" s="23" t="s">
         <v>59</v>
       </c>
@@ -23434,7 +23484,7 @@
       </c>
       <c r="Q159" s="17"/>
     </row>
-    <row r="160" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" s="23" t="s">
         <v>60</v>
       </c>
@@ -23479,7 +23529,7 @@
       </c>
       <c r="Q160" s="17"/>
     </row>
-    <row r="161" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" s="23" t="s">
         <v>61</v>
       </c>
@@ -23524,7 +23574,7 @@
       </c>
       <c r="Q161" s="17"/>
     </row>
-    <row r="162" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" s="23" t="s">
         <v>62</v>
       </c>
@@ -23569,7 +23619,7 @@
       </c>
       <c r="Q162" s="17"/>
     </row>
-    <row r="163" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" s="23" t="s">
         <v>63</v>
       </c>
@@ -23614,7 +23664,7 @@
       </c>
       <c r="Q163" s="17"/>
     </row>
-    <row r="164" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" s="23" t="s">
         <v>87</v>
       </c>
@@ -23659,7 +23709,7 @@
       </c>
       <c r="Q164" s="17"/>
     </row>
-    <row r="165" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" s="23" t="s">
         <v>90</v>
       </c>
@@ -23704,7 +23754,7 @@
       </c>
       <c r="Q165" s="17"/>
     </row>
-    <row r="166" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" s="23" t="s">
         <v>91</v>
       </c>
@@ -23749,7 +23799,7 @@
       </c>
       <c r="Q166" s="17"/>
     </row>
-    <row r="167" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" s="23" t="s">
         <v>92</v>
       </c>
@@ -23794,7 +23844,7 @@
       </c>
       <c r="Q167" s="17"/>
     </row>
-    <row r="168" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" s="23" t="s">
         <v>93</v>
       </c>
@@ -23839,7 +23889,7 @@
       </c>
       <c r="Q168" s="17"/>
     </row>
-    <row r="169" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" s="23" t="s">
         <v>94</v>
       </c>
@@ -23884,7 +23934,7 @@
       </c>
       <c r="Q169" s="17"/>
     </row>
-    <row r="170" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" s="23" t="s">
         <v>95</v>
       </c>
@@ -23929,7 +23979,7 @@
       </c>
       <c r="Q170" s="17"/>
     </row>
-    <row r="171" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" s="23" t="s">
         <v>220</v>
       </c>
@@ -23974,7 +24024,7 @@
       </c>
       <c r="Q171" s="17"/>
     </row>
-    <row r="172" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" s="23" t="s">
         <v>223</v>
       </c>
@@ -24019,7 +24069,7 @@
       </c>
       <c r="Q172" s="17"/>
     </row>
-    <row r="173" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" s="23" t="s">
         <v>224</v>
       </c>
@@ -24064,7 +24114,7 @@
       </c>
       <c r="Q173" s="17"/>
     </row>
-    <row r="174" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" s="23" t="s">
         <v>225</v>
       </c>
@@ -24466,7 +24516,7 @@
       </c>
       <c r="Q181" s="17"/>
     </row>
-    <row r="182" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" s="23" t="s">
         <v>219</v>
       </c>
@@ -24511,7 +24561,7 @@
       </c>
       <c r="Q182" s="17"/>
     </row>
-    <row r="183" spans="1:17" ht="21.4" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:17" ht="21.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" s="23" t="s">
         <v>64</v>
       </c>
@@ -25072,6 +25122,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:Q193" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N193">
     <sortCondition ref="A2:A193"/>
   </sortState>
@@ -35129,34 +35186,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="14.65" x14ac:dyDescent="0.45">
-      <c r="A1" s="159" t="s">
+      <c r="A1" s="160" t="s">
         <v>1170</v>
       </c>
-      <c r="B1" s="159" t="s">
+      <c r="B1" s="160" t="s">
         <v>1171</v>
       </c>
-      <c r="C1" s="159" t="s">
+      <c r="C1" s="160" t="s">
         <v>1172</v>
       </c>
-      <c r="D1" s="160" t="s">
+      <c r="D1" s="161" t="s">
         <v>1173</v>
       </c>
-      <c r="E1" s="160"/>
-      <c r="F1" s="160"/>
-      <c r="G1" s="160" t="s">
+      <c r="E1" s="161"/>
+      <c r="F1" s="161"/>
+      <c r="G1" s="161" t="s">
         <v>1174</v>
       </c>
-      <c r="H1" s="160"/>
-      <c r="I1" s="160"/>
+      <c r="H1" s="161"/>
+      <c r="I1" s="161"/>
       <c r="J1" s="108"/>
       <c r="K1" s="109" t="s">
         <v>1175</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="14.65" x14ac:dyDescent="0.45">
-      <c r="A2" s="159"/>
-      <c r="B2" s="159"/>
-      <c r="C2" s="159"/>
+      <c r="A2" s="160"/>
+      <c r="B2" s="160"/>
+      <c r="C2" s="160"/>
       <c r="D2" s="107" t="s">
         <v>1176</v>
       </c>
@@ -37676,19 +37733,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="14.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="159" t="s">
+      <c r="A1" s="160" t="s">
         <v>1197</v>
       </c>
-      <c r="B1" s="159"/>
-      <c r="C1" s="159"/>
-      <c r="D1" s="159"/>
-      <c r="E1" s="159"/>
-      <c r="F1" s="159"/>
-      <c r="G1" s="159"/>
-      <c r="H1" s="159"/>
-      <c r="I1" s="159"/>
-      <c r="J1" s="159"/>
-      <c r="K1" s="159"/>
+      <c r="B1" s="160"/>
+      <c r="C1" s="160"/>
+      <c r="D1" s="160"/>
+      <c r="E1" s="160"/>
+      <c r="F1" s="160"/>
+      <c r="G1" s="160"/>
+      <c r="H1" s="160"/>
+      <c r="I1" s="160"/>
+      <c r="J1" s="160"/>
+      <c r="K1" s="160"/>
     </row>
     <row r="2" spans="1:11" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A2" s="134" t="s">
@@ -38421,16 +38478,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="159" t="s">
+      <c r="A1" s="160" t="s">
         <v>1198</v>
       </c>
-      <c r="B1" s="159"/>
-      <c r="C1" s="159"/>
-      <c r="D1" s="159"/>
-      <c r="E1" s="159"/>
-      <c r="F1" s="159"/>
-      <c r="G1" s="159"/>
-      <c r="H1" s="159"/>
+      <c r="B1" s="160"/>
+      <c r="C1" s="160"/>
+      <c r="D1" s="160"/>
+      <c r="E1" s="160"/>
+      <c r="F1" s="160"/>
+      <c r="G1" s="160"/>
+      <c r="H1" s="160"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A2" s="150" t="s">

</xml_diff>

<commit_message>
new elec meters installed
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2772" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62980A75-8457-4502-B976-4FDC60B88EDD}"/>
+  <xr:revisionPtr revIDLastSave="2790" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C34928C-039F-478B-A0BD-B91D78B154EC}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-7455" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="21720" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FS Elec" sheetId="4" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5044" uniqueCount="1204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5050" uniqueCount="1204">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -12939,7 +12939,9 @@
       <c r="B141" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C141" s="2"/>
+      <c r="C141" s="2">
+        <v>14558069556</v>
+      </c>
       <c r="D141" s="2">
         <v>71205556</v>
       </c>
@@ -12952,14 +12954,18 @@
       <c r="G141" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H141" s="2"/>
+      <c r="H141" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="I141" s="30" t="s">
         <v>36</v>
       </c>
       <c r="J141" s="9">
         <v>0</v>
       </c>
-      <c r="K141" s="2"/>
+      <c r="K141" s="4">
+        <v>46224</v>
+      </c>
       <c r="L141" s="11" t="b">
         <v>0</v>
       </c>
@@ -12987,7 +12993,9 @@
       <c r="B142" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C142" s="2"/>
+      <c r="C142" s="2">
+        <v>14558069721</v>
+      </c>
       <c r="D142" s="2">
         <v>71205556</v>
       </c>
@@ -13000,14 +13008,18 @@
       <c r="G142" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H142" s="2"/>
+      <c r="H142" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="I142" s="30" t="s">
         <v>36</v>
       </c>
       <c r="J142" s="9">
         <v>0</v>
       </c>
-      <c r="K142" s="2"/>
+      <c r="K142" s="4">
+        <v>46224</v>
+      </c>
       <c r="L142" s="11" t="b">
         <v>0</v>
       </c>
@@ -13035,7 +13047,9 @@
       <c r="B143" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C143" s="2"/>
+      <c r="C143" s="2">
+        <v>14558068038</v>
+      </c>
       <c r="D143" s="2">
         <v>71205556</v>
       </c>
@@ -13048,14 +13062,18 @@
       <c r="G143" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H143" s="2"/>
+      <c r="H143" s="8" t="s">
+        <v>33</v>
+      </c>
       <c r="I143" s="30" t="s">
         <v>36</v>
       </c>
       <c r="J143" s="9">
         <v>0</v>
       </c>
-      <c r="K143" s="2"/>
+      <c r="K143" s="4">
+        <v>46224</v>
+      </c>
       <c r="L143" s="11" t="b">
         <v>0</v>
       </c>
@@ -13083,7 +13101,9 @@
       <c r="B144" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C144" s="2"/>
+      <c r="C144" s="2">
+        <v>14558069135</v>
+      </c>
       <c r="D144" s="2">
         <v>71205556</v>
       </c>
@@ -13096,14 +13116,18 @@
       <c r="G144" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H144" s="2"/>
+      <c r="H144" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="I144" s="30" t="s">
         <v>36</v>
       </c>
       <c r="J144" s="9">
         <v>0</v>
       </c>
-      <c r="K144" s="2"/>
+      <c r="K144" s="4">
+        <v>46224</v>
+      </c>
       <c r="L144" s="11" t="b">
         <v>0</v>
       </c>
@@ -13131,7 +13155,9 @@
       <c r="B145" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C145" s="2"/>
+      <c r="C145" s="2">
+        <v>14558068103</v>
+      </c>
       <c r="D145" s="2">
         <v>71205556</v>
       </c>
@@ -13144,14 +13170,18 @@
       <c r="G145" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H145" s="2"/>
+      <c r="H145" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="I145" s="30" t="s">
         <v>36</v>
       </c>
       <c r="J145" s="9">
         <v>0</v>
       </c>
-      <c r="K145" s="2"/>
+      <c r="K145" s="4">
+        <v>46224</v>
+      </c>
       <c r="L145" s="11" t="b">
         <v>0</v>
       </c>
@@ -13287,7 +13317,9 @@
       <c r="B148" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C148" s="2"/>
+      <c r="C148" s="2">
+        <v>14558069838</v>
+      </c>
       <c r="D148" s="2">
         <v>71205556</v>
       </c>
@@ -13300,14 +13332,18 @@
       <c r="G148" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H148" s="2"/>
+      <c r="H148" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="I148" s="30" t="s">
         <v>36</v>
       </c>
       <c r="J148" s="9">
         <v>0</v>
       </c>
-      <c r="K148" s="2"/>
+      <c r="K148" s="4">
+        <v>46224</v>
+      </c>
       <c r="L148" s="11" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
new kamstrup water meters installed
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3174" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F006E32E-8FEA-41DD-A5AF-33F38E2021F9}"/>
+  <xr:revisionPtr revIDLastSave="3257" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FAAA7020-BD77-4218-87E5-37DA3159A5A7}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="59280" yWindow="-2430" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FS Elec" sheetId="4" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FS Elec'!$A$1:$U$192</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'FS Water'!$A$1:$S$193</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4942" uniqueCount="1236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4959" uniqueCount="1253">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -3753,6 +3753,57 @@
   </si>
   <si>
     <t>2cf7f1207310074f</t>
+  </si>
+  <si>
+    <t>54789040</t>
+  </si>
+  <si>
+    <t>54789077</t>
+  </si>
+  <si>
+    <t>54789045</t>
+  </si>
+  <si>
+    <t>54789042</t>
+  </si>
+  <si>
+    <t>54789038</t>
+  </si>
+  <si>
+    <t>54789034</t>
+  </si>
+  <si>
+    <t>54789048</t>
+  </si>
+  <si>
+    <t>54789039</t>
+  </si>
+  <si>
+    <t>54789037</t>
+  </si>
+  <si>
+    <t>54789036</t>
+  </si>
+  <si>
+    <t>54789041</t>
+  </si>
+  <si>
+    <t>54789044</t>
+  </si>
+  <si>
+    <t>54789047</t>
+  </si>
+  <si>
+    <t>54789035</t>
+  </si>
+  <si>
+    <t>54789046</t>
+  </si>
+  <si>
+    <t>54789043</t>
+  </si>
+  <si>
+    <t>54789074</t>
   </si>
 </sst>
 </file>
@@ -4796,13 +4847,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -16882,7 +16933,7 @@
       <c r="L192" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M192" s="143" t="s">
+      <c r="M192" s="141" t="s">
         <v>1235</v>
       </c>
       <c r="N192" s="134">
@@ -16936,8 +16987,8 @@
     <col min="5" max="5" width="19.73046875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25.59765625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31.1328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.46484375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.46484375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="39.53125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28.86328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="27.3984375" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="20.265625" customWidth="1"/>
     <col min="14" max="14" width="35.46484375" customWidth="1"/>
@@ -17954,18 +18005,24 @@
       <c r="B22" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="C22" s="53"/>
+      <c r="C22" s="53" t="s">
+        <v>1252</v>
+      </c>
       <c r="D22" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E22" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F22" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
+      <c r="G22" s="3">
+        <v>0.11799999999999999</v>
+      </c>
+      <c r="H22" s="57">
+        <v>46248</v>
+      </c>
       <c r="I22" s="21" t="b">
         <v>0</v>
       </c>
@@ -18048,18 +18105,24 @@
       <c r="B24" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="53"/>
+      <c r="C24" s="53" t="s">
+        <v>1251</v>
+      </c>
       <c r="D24" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E24" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F24" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
+      <c r="G24" s="3">
+        <v>0.151</v>
+      </c>
+      <c r="H24" s="57">
+        <v>46248</v>
+      </c>
       <c r="I24" s="21" t="b">
         <v>0</v>
       </c>
@@ -18424,18 +18487,24 @@
       <c r="B32" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="C32" s="53"/>
+      <c r="C32" s="53" t="s">
+        <v>1250</v>
+      </c>
       <c r="D32" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E32" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F32" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
+      <c r="G32" s="3">
+        <v>0.12</v>
+      </c>
+      <c r="H32" s="57">
+        <v>46248</v>
+      </c>
       <c r="I32" s="21" t="b">
         <v>0</v>
       </c>
@@ -18471,18 +18540,24 @@
       <c r="B33" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C33" s="53"/>
+      <c r="C33" s="53" t="s">
+        <v>1243</v>
+      </c>
       <c r="D33" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E33" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F33" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
+      <c r="G33" s="3">
+        <v>0.151</v>
+      </c>
+      <c r="H33" s="57">
+        <v>46248</v>
+      </c>
       <c r="I33" s="21" t="b">
         <v>0</v>
       </c>
@@ -18518,18 +18593,24 @@
       <c r="B34" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C34" s="53"/>
+      <c r="C34" s="53" t="s">
+        <v>1242</v>
+      </c>
       <c r="D34" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E34" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F34" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
+      <c r="G34" s="3">
+        <v>0.12</v>
+      </c>
+      <c r="H34" s="57">
+        <v>46248</v>
+      </c>
       <c r="I34" s="21" t="b">
         <v>0</v>
       </c>
@@ -25292,18 +25373,24 @@
       <c r="B164" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C164" s="53"/>
+      <c r="C164" s="53" t="s">
+        <v>1241</v>
+      </c>
       <c r="D164" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E164" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F164" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G164" s="3"/>
-      <c r="H164" s="3"/>
+      <c r="G164" s="3">
+        <v>0.153</v>
+      </c>
+      <c r="H164" s="57">
+        <v>46248</v>
+      </c>
       <c r="I164" s="21" t="b">
         <v>0</v>
       </c>
@@ -25339,18 +25426,24 @@
       <c r="B165" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C165" s="53"/>
+      <c r="C165" s="53" t="s">
+        <v>1240</v>
+      </c>
       <c r="D165" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E165" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F165" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G165" s="3"/>
-      <c r="H165" s="3"/>
+      <c r="G165" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="H165" s="57">
+        <v>46248</v>
+      </c>
       <c r="I165" s="21" t="b">
         <v>0</v>
       </c>
@@ -25386,18 +25479,24 @@
       <c r="B166" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C166" s="53"/>
+      <c r="C166" s="53" t="s">
+        <v>1239</v>
+      </c>
       <c r="D166" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E166" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F166" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G166" s="3"/>
-      <c r="H166" s="3"/>
+      <c r="G166" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="H166" s="57">
+        <v>46248</v>
+      </c>
       <c r="I166" s="21" t="b">
         <v>0</v>
       </c>
@@ -25433,18 +25532,24 @@
       <c r="B167" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C167" s="53"/>
+      <c r="C167" s="53" t="s">
+        <v>1238</v>
+      </c>
       <c r="D167" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E167" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F167" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G167" s="3"/>
-      <c r="H167" s="3"/>
+      <c r="G167" s="3">
+        <v>0.12</v>
+      </c>
+      <c r="H167" s="57">
+        <v>46248</v>
+      </c>
       <c r="I167" s="21" t="b">
         <v>0</v>
       </c>
@@ -25480,18 +25585,24 @@
       <c r="B168" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C168" s="53"/>
+      <c r="C168" s="53" t="s">
+        <v>1237</v>
+      </c>
       <c r="D168" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E168" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F168" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G168" s="3"/>
-      <c r="H168" s="3"/>
+      <c r="G168" s="3">
+        <v>0.11700000000000001</v>
+      </c>
+      <c r="H168" s="57">
+        <v>46248</v>
+      </c>
       <c r="I168" s="21" t="b">
         <v>0</v>
       </c>
@@ -25527,18 +25638,24 @@
       <c r="B169" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C169" s="53"/>
+      <c r="C169" s="53" t="s">
+        <v>1236</v>
+      </c>
       <c r="D169" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E169" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F169" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G169" s="3"/>
-      <c r="H169" s="3"/>
+      <c r="G169" s="3">
+        <v>0.151</v>
+      </c>
+      <c r="H169" s="57">
+        <v>46248</v>
+      </c>
       <c r="I169" s="21" t="b">
         <v>0</v>
       </c>
@@ -25621,18 +25738,24 @@
       <c r="B171" s="59" t="s">
         <v>65</v>
       </c>
-      <c r="C171" s="53"/>
+      <c r="C171" s="53" t="s">
+        <v>1247</v>
+      </c>
       <c r="D171" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E171" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F171" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G171" s="3"/>
-      <c r="H171" s="3"/>
+      <c r="G171" s="3">
+        <v>0.121</v>
+      </c>
+      <c r="H171" s="57">
+        <v>46248</v>
+      </c>
       <c r="I171" s="21" t="b">
         <v>0</v>
       </c>
@@ -25668,18 +25791,24 @@
       <c r="B172" s="59" t="s">
         <v>65</v>
       </c>
-      <c r="C172" s="53"/>
+      <c r="C172" s="53" t="s">
+        <v>1244</v>
+      </c>
       <c r="D172" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E172" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F172" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G172" s="3"/>
-      <c r="H172" s="3"/>
+      <c r="G172" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="H172" s="57">
+        <v>46248</v>
+      </c>
       <c r="I172" s="21" t="b">
         <v>0</v>
       </c>
@@ -25715,18 +25844,24 @@
       <c r="B173" s="59" t="s">
         <v>65</v>
       </c>
-      <c r="C173" s="53"/>
+      <c r="C173" s="53" t="s">
+        <v>1245</v>
+      </c>
       <c r="D173" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E173" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F173" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G173" s="3"/>
-      <c r="H173" s="3"/>
+      <c r="G173" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="H173" s="57">
+        <v>46248</v>
+      </c>
       <c r="I173" s="21" t="b">
         <v>0</v>
       </c>
@@ -25762,18 +25897,24 @@
       <c r="B174" s="59" t="s">
         <v>65</v>
       </c>
-      <c r="C174" s="53"/>
+      <c r="C174" s="53" t="s">
+        <v>1246</v>
+      </c>
       <c r="D174" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E174" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F174" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G174" s="3"/>
-      <c r="H174" s="3"/>
+      <c r="G174" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="H174" s="57">
+        <v>46248</v>
+      </c>
       <c r="I174" s="21" t="b">
         <v>0</v>
       </c>
@@ -26180,18 +26321,24 @@
       <c r="B182" s="59" t="s">
         <v>65</v>
       </c>
-      <c r="C182" s="53"/>
+      <c r="C182" s="53" t="s">
+        <v>1248</v>
+      </c>
       <c r="D182" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E182" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F182" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G182" s="3"/>
-      <c r="H182" s="3"/>
+      <c r="G182" s="3">
+        <v>0.12</v>
+      </c>
+      <c r="H182" s="57">
+        <v>46248</v>
+      </c>
       <c r="I182" s="21" t="b">
         <v>0</v>
       </c>
@@ -26227,18 +26374,24 @@
       <c r="B183" s="59" t="s">
         <v>65</v>
       </c>
-      <c r="C183" s="53"/>
+      <c r="C183" s="53" t="s">
+        <v>1249</v>
+      </c>
       <c r="D183" s="53" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="E183" s="53" t="s">
-        <v>285</v>
+        <v>357</v>
       </c>
       <c r="F183" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G183" s="3"/>
-      <c r="H183" s="3"/>
+      <c r="G183" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="H183" s="57">
+        <v>46248</v>
+      </c>
       <c r="I183" s="21" t="b">
         <v>0</v>
       </c>
@@ -36860,34 +37013,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="14.65" x14ac:dyDescent="0.45">
-      <c r="A1" s="141" t="s">
+      <c r="A1" s="142" t="s">
         <v>1170</v>
       </c>
-      <c r="B1" s="141" t="s">
+      <c r="B1" s="142" t="s">
         <v>1171</v>
       </c>
-      <c r="C1" s="141" t="s">
+      <c r="C1" s="142" t="s">
         <v>1172</v>
       </c>
-      <c r="D1" s="142" t="s">
+      <c r="D1" s="143" t="s">
         <v>1173</v>
       </c>
-      <c r="E1" s="142"/>
-      <c r="F1" s="142"/>
-      <c r="G1" s="142" t="s">
+      <c r="E1" s="143"/>
+      <c r="F1" s="143"/>
+      <c r="G1" s="143" t="s">
         <v>1174</v>
       </c>
-      <c r="H1" s="142"/>
-      <c r="I1" s="142"/>
+      <c r="H1" s="143"/>
+      <c r="I1" s="143"/>
       <c r="J1" s="108"/>
       <c r="K1" s="109" t="s">
         <v>1175</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="14.65" x14ac:dyDescent="0.45">
-      <c r="A2" s="141"/>
-      <c r="B2" s="141"/>
-      <c r="C2" s="141"/>
+      <c r="A2" s="142"/>
+      <c r="B2" s="142"/>
+      <c r="C2" s="142"/>
       <c r="D2" s="107" t="s">
         <v>1176</v>
       </c>

</xml_diff>

<commit_message>
new water meters, and elec AMR installed
</commit_message>
<xml_diff>
--- a/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
+++ b/EVG_SIT_FS_Meter_Commissioning_2026-07-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Evergreen/Evergreen Sitari/Site initialization/Freestanding/EVG_FS_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3417" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F88C7F61-75C8-4ABB-B71B-665CB30D1C32}"/>
+  <xr:revisionPtr revIDLastSave="3549" documentId="8_{C97FC332-2E41-401D-B97C-40A4EC775E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9DEF16A-C557-4089-9CFF-8B4A4B172C5F}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-11010" windowWidth="16440" windowHeight="28320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="88080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FS Elec" sheetId="4" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4986" uniqueCount="1278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5061" uniqueCount="1292">
   <si>
     <t xml:space="preserve">Stand Number </t>
   </si>
@@ -3879,6 +3879,48 @@
   </si>
   <si>
     <t>10596189</t>
+  </si>
+  <si>
+    <t>10596229</t>
+  </si>
+  <si>
+    <t>10596237</t>
+  </si>
+  <si>
+    <t>10596377</t>
+  </si>
+  <si>
+    <t>10596304</t>
+  </si>
+  <si>
+    <t>10596231</t>
+  </si>
+  <si>
+    <t>2cf7f12072903411</t>
+  </si>
+  <si>
+    <t>2cf7f12072903bab</t>
+  </si>
+  <si>
+    <t>2cf7f120729018c1</t>
+  </si>
+  <si>
+    <t>2cf7f12072902fd1</t>
+  </si>
+  <si>
+    <t>2cf7f12072903b79</t>
+  </si>
+  <si>
+    <t>2cf7f120731008bf</t>
+  </si>
+  <si>
+    <t>2cf7f12072902d12</t>
+  </si>
+  <si>
+    <t>2cf7f12072901d88</t>
+  </si>
+  <si>
+    <t>2cf7f12072901e3a</t>
   </si>
 </sst>
 </file>
@@ -5418,7 +5460,8 @@
     <col min="9" max="9" width="16.59765625" style="5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="26.3984375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="27.265625" style="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="16.59765625" customWidth="1"/>
+    <col min="12" max="12" width="16.59765625" customWidth="1"/>
+    <col min="13" max="13" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="9.3984375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17.3984375" bestFit="1" customWidth="1"/>
     <col min="16" max="19" width="11.265625" bestFit="1" customWidth="1"/>
@@ -5526,10 +5569,14 @@
         <v>46206</v>
       </c>
       <c r="L2" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>1286</v>
+      </c>
+      <c r="N2" s="2">
+        <v>6</v>
+      </c>
       <c r="O2" s="64" t="s">
         <v>25</v>
       </c>
@@ -5583,10 +5630,14 @@
         <v>46206</v>
       </c>
       <c r="L3" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>1286</v>
+      </c>
+      <c r="N3" s="2">
+        <v>3</v>
+      </c>
       <c r="O3" s="64" t="s">
         <v>28</v>
       </c>
@@ -5640,10 +5691,14 @@
         <v>46206</v>
       </c>
       <c r="L4" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>1286</v>
+      </c>
+      <c r="N4" s="2">
+        <v>5</v>
+      </c>
       <c r="O4" s="64" t="s">
         <v>25</v>
       </c>
@@ -5697,10 +5752,14 @@
         <v>46206</v>
       </c>
       <c r="L5" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>1286</v>
+      </c>
+      <c r="N5" s="2">
+        <v>2</v>
+      </c>
       <c r="O5" s="64" t="s">
         <v>28</v>
       </c>
@@ -5754,10 +5813,14 @@
         <v>46206</v>
       </c>
       <c r="L6" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>1286</v>
+      </c>
+      <c r="N6" s="2">
+        <v>4</v>
+      </c>
       <c r="O6" s="64" t="s">
         <v>25</v>
       </c>
@@ -5811,10 +5874,14 @@
         <v>46206</v>
       </c>
       <c r="L7" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>1286</v>
+      </c>
+      <c r="N7" s="2">
+        <v>1</v>
+      </c>
       <c r="O7" s="64" t="s">
         <v>28</v>
       </c>
@@ -5870,8 +5937,10 @@
       <c r="L8" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
+      <c r="M8" s="2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="N8" s="7"/>
       <c r="O8" s="64" t="s">
         <v>37</v>
       </c>
@@ -5927,8 +5996,10 @@
       <c r="L9" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
+      <c r="M9" s="2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="N9" s="7"/>
       <c r="O9" s="64" t="s">
         <v>39</v>
       </c>
@@ -5984,8 +6055,10 @@
       <c r="L10" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
+      <c r="M10" s="2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="N10" s="7"/>
       <c r="O10" s="64" t="s">
         <v>37</v>
       </c>
@@ -6041,8 +6114,10 @@
       <c r="L11" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
+      <c r="M11" s="2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="N11" s="7"/>
       <c r="O11" s="64" t="s">
         <v>39</v>
       </c>
@@ -6098,8 +6173,10 @@
       <c r="L12" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
+      <c r="M12" s="2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="N12" s="7"/>
       <c r="O12" s="64" t="s">
         <v>37</v>
       </c>
@@ -6155,8 +6232,10 @@
       <c r="L13" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
+      <c r="M13" s="2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="N13" s="7"/>
       <c r="O13" s="64" t="s">
         <v>39</v>
       </c>
@@ -6212,8 +6291,10 @@
       <c r="L14" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
+      <c r="M14" s="2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="N14" s="7"/>
       <c r="O14" s="64" t="s">
         <v>39</v>
       </c>
@@ -6269,8 +6350,10 @@
       <c r="L15" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
+      <c r="M15" s="2" t="s">
+        <v>1290</v>
+      </c>
+      <c r="N15" s="7"/>
       <c r="O15" s="64" t="s">
         <v>37</v>
       </c>
@@ -6326,8 +6409,10 @@
       <c r="L16" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
+      <c r="M16" s="2" t="s">
+        <v>1290</v>
+      </c>
+      <c r="N16" s="7"/>
       <c r="O16" s="64" t="s">
         <v>37</v>
       </c>
@@ -6383,8 +6468,10 @@
       <c r="L17" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
+      <c r="M17" s="2" t="s">
+        <v>1290</v>
+      </c>
+      <c r="N17" s="7"/>
       <c r="O17" s="64" t="s">
         <v>39</v>
       </c>
@@ -6440,8 +6527,10 @@
       <c r="L18" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
+      <c r="M18" s="2" t="s">
+        <v>1290</v>
+      </c>
+      <c r="N18" s="7"/>
       <c r="O18" s="64" t="s">
         <v>37</v>
       </c>
@@ -6497,8 +6586,10 @@
       <c r="L19" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
+      <c r="M19" s="2" t="s">
+        <v>1290</v>
+      </c>
+      <c r="N19" s="7"/>
       <c r="O19" s="64" t="s">
         <v>39</v>
       </c>
@@ -6554,8 +6645,10 @@
       <c r="L20" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
+      <c r="M20" s="2" t="s">
+        <v>1290</v>
+      </c>
+      <c r="N20" s="7"/>
       <c r="O20" s="64" t="s">
         <v>37</v>
       </c>
@@ -6611,8 +6704,10 @@
       <c r="L21" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
+      <c r="M21" s="2" t="s">
+        <v>1290</v>
+      </c>
+      <c r="N21" s="7"/>
       <c r="O21" s="64" t="s">
         <v>39</v>
       </c>
@@ -6668,8 +6763,10 @@
       <c r="L22" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
+      <c r="M22" s="2" t="s">
+        <v>1290</v>
+      </c>
+      <c r="N22" s="7"/>
       <c r="O22" s="64" t="s">
         <v>39</v>
       </c>
@@ -6725,8 +6822,10 @@
       <c r="L23" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2">
+      <c r="M23" s="2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="N23" s="7">
         <v>1</v>
       </c>
       <c r="O23" s="64" t="s">
@@ -6784,8 +6883,10 @@
       <c r="L24" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2">
+      <c r="M24" s="2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="N24" s="7">
         <v>7</v>
       </c>
       <c r="O24" s="64" t="s">
@@ -6843,8 +6944,10 @@
       <c r="L25" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2">
+      <c r="M25" s="2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="N25" s="7">
         <v>2</v>
       </c>
       <c r="O25" s="64" t="s">
@@ -6902,8 +7005,10 @@
       <c r="L26" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2">
+      <c r="M26" s="2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="N26" s="7">
         <v>3</v>
       </c>
       <c r="O26" s="64" t="s">
@@ -6961,8 +7066,10 @@
       <c r="L27" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M27" s="2"/>
-      <c r="N27" s="2">
+      <c r="M27" s="2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="N27" s="7">
         <v>8</v>
       </c>
       <c r="O27" s="64" t="s">
@@ -7020,8 +7127,10 @@
       <c r="L28" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M28" s="2"/>
-      <c r="N28" s="2">
+      <c r="M28" s="2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="N28" s="7">
         <v>4</v>
       </c>
       <c r="O28" s="64" t="s">
@@ -7079,8 +7188,10 @@
       <c r="L29" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M29" s="2"/>
-      <c r="N29" s="2">
+      <c r="M29" s="2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="N29" s="7">
         <v>5</v>
       </c>
       <c r="O29" s="64" t="s">
@@ -7138,8 +7249,10 @@
       <c r="L30" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2">
+      <c r="M30" s="2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="N30" s="7">
         <v>6</v>
       </c>
       <c r="O30" s="64" t="s">
@@ -7200,7 +7313,7 @@
       <c r="M31" s="2" t="s">
         <v>1214</v>
       </c>
-      <c r="N31" s="2">
+      <c r="N31" s="7">
         <v>1</v>
       </c>
       <c r="O31" s="64" t="s">
@@ -7261,7 +7374,7 @@
       <c r="M32" s="2" t="s">
         <v>1214</v>
       </c>
-      <c r="N32" s="2">
+      <c r="N32" s="7">
         <v>2</v>
       </c>
       <c r="O32" s="64" t="s">
@@ -7322,7 +7435,7 @@
       <c r="M33" s="2" t="s">
         <v>1214</v>
       </c>
-      <c r="N33" s="2">
+      <c r="N33" s="7">
         <v>3</v>
       </c>
       <c r="O33" s="64" t="s">
@@ -7383,7 +7496,7 @@
       <c r="M34" s="2" t="s">
         <v>1214</v>
       </c>
-      <c r="N34" s="2">
+      <c r="N34" s="7">
         <v>4</v>
       </c>
       <c r="O34" s="64" t="s">
@@ -7566,7 +7679,7 @@
       <c r="M37" s="2" t="s">
         <v>1215</v>
       </c>
-      <c r="N37" s="2">
+      <c r="N37" s="7">
         <v>9</v>
       </c>
       <c r="O37" s="64" t="s">
@@ -7627,7 +7740,7 @@
       <c r="M38" s="2" t="s">
         <v>1215</v>
       </c>
-      <c r="N38" s="2">
+      <c r="N38" s="7">
         <v>6</v>
       </c>
       <c r="O38" s="64" t="s">
@@ -7753,7 +7866,7 @@
       <c r="M40" s="2" t="s">
         <v>1215</v>
       </c>
-      <c r="N40" s="2">
+      <c r="N40" s="7">
         <v>5</v>
       </c>
       <c r="O40" s="64" t="s">
@@ -7879,7 +7992,7 @@
       <c r="M42" s="2" t="s">
         <v>1215</v>
       </c>
-      <c r="N42" s="2">
+      <c r="N42" s="7">
         <v>4</v>
       </c>
       <c r="O42" s="64" t="s">
@@ -7940,7 +8053,7 @@
       <c r="M43" s="2" t="s">
         <v>1215</v>
       </c>
-      <c r="N43" s="2">
+      <c r="N43" s="7">
         <v>3</v>
       </c>
       <c r="O43" s="64" t="s">
@@ -8001,7 +8114,7 @@
       <c r="M44" s="2" t="s">
         <v>1215</v>
       </c>
-      <c r="N44" s="2">
+      <c r="N44" s="7">
         <v>2</v>
       </c>
       <c r="O44" s="64" t="s">
@@ -8120,8 +8233,10 @@
       <c r="L46" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M46" s="2"/>
-      <c r="N46" s="2">
+      <c r="M46" s="2" t="s">
+        <v>1283</v>
+      </c>
+      <c r="N46" s="7">
         <v>6</v>
       </c>
       <c r="O46" s="64" t="s">
@@ -8179,8 +8294,10 @@
       <c r="L47" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M47" s="2"/>
-      <c r="N47" s="2">
+      <c r="M47" s="2" t="s">
+        <v>1283</v>
+      </c>
+      <c r="N47" s="7">
         <v>3</v>
       </c>
       <c r="O47" s="64" t="s">
@@ -8238,8 +8355,10 @@
       <c r="L48" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M48" s="2"/>
-      <c r="N48" s="2">
+      <c r="M48" s="2" t="s">
+        <v>1283</v>
+      </c>
+      <c r="N48" s="7">
         <v>2</v>
       </c>
       <c r="O48" s="64" t="s">
@@ -8297,8 +8416,10 @@
       <c r="L49" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M49" s="2"/>
-      <c r="N49" s="2">
+      <c r="M49" s="2" t="s">
+        <v>1283</v>
+      </c>
+      <c r="N49" s="7">
         <v>1</v>
       </c>
       <c r="O49" s="64" t="s">
@@ -8356,8 +8477,10 @@
       <c r="L50" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M50" s="2"/>
-      <c r="N50" s="2">
+      <c r="M50" s="2" t="s">
+        <v>1283</v>
+      </c>
+      <c r="N50" s="7">
         <v>5</v>
       </c>
       <c r="O50" s="64" t="s">
@@ -8415,8 +8538,10 @@
       <c r="L51" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M51" s="2"/>
-      <c r="N51" s="2">
+      <c r="M51" s="2" t="s">
+        <v>1283</v>
+      </c>
+      <c r="N51" s="7">
         <v>7</v>
       </c>
       <c r="O51" s="64" t="s">
@@ -8474,8 +8599,10 @@
       <c r="L52" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M52" s="2"/>
-      <c r="N52" s="2">
+      <c r="M52" s="2" t="s">
+        <v>1283</v>
+      </c>
+      <c r="N52" s="7">
         <v>4</v>
       </c>
       <c r="O52" s="64" t="s">
@@ -9044,7 +9171,7 @@
       <c r="M61" s="2" t="s">
         <v>1217</v>
       </c>
-      <c r="N61" s="2">
+      <c r="N61" s="7">
         <v>9</v>
       </c>
       <c r="O61" s="64" t="s">
@@ -9105,7 +9232,7 @@
       <c r="M62" s="2" t="s">
         <v>1217</v>
       </c>
-      <c r="N62" s="2">
+      <c r="N62" s="7">
         <v>8</v>
       </c>
       <c r="O62" s="64" t="s">
@@ -9292,7 +9419,7 @@
       <c r="M65" s="2" t="s">
         <v>1217</v>
       </c>
-      <c r="N65" s="2">
+      <c r="N65" s="7">
         <v>6</v>
       </c>
       <c r="O65" s="64" t="s">
@@ -9418,7 +9545,7 @@
       <c r="M67" s="2" t="s">
         <v>1217</v>
       </c>
-      <c r="N67" s="2">
+      <c r="N67" s="7">
         <v>5</v>
       </c>
       <c r="O67" s="64" t="s">
@@ -9609,7 +9736,7 @@
       <c r="M70" s="2" t="s">
         <v>1218</v>
       </c>
-      <c r="N70" s="2">
+      <c r="N70" s="7">
         <v>1</v>
       </c>
       <c r="O70" s="64" t="s">
@@ -9670,7 +9797,7 @@
       <c r="M71" s="2" t="s">
         <v>1218</v>
       </c>
-      <c r="N71" s="2">
+      <c r="N71" s="7">
         <v>2</v>
       </c>
       <c r="O71" s="64" t="s">
@@ -9731,7 +9858,7 @@
       <c r="M72" s="2" t="s">
         <v>1218</v>
       </c>
-      <c r="N72" s="2">
+      <c r="N72" s="7">
         <v>6</v>
       </c>
       <c r="O72" s="64" t="s">
@@ -9792,7 +9919,7 @@
       <c r="M73" s="2" t="s">
         <v>1218</v>
       </c>
-      <c r="N73" s="2">
+      <c r="N73" s="7">
         <v>3</v>
       </c>
       <c r="O73" s="64" t="s">
@@ -9853,7 +9980,7 @@
       <c r="M74" s="2" t="s">
         <v>1218</v>
       </c>
-      <c r="N74" s="2">
+      <c r="N74" s="7">
         <v>7</v>
       </c>
       <c r="O74" s="64" t="s">
@@ -9914,7 +10041,7 @@
       <c r="M75" s="2" t="s">
         <v>1218</v>
       </c>
-      <c r="N75" s="2">
+      <c r="N75" s="7">
         <v>4</v>
       </c>
       <c r="O75" s="64" t="s">
@@ -9975,7 +10102,7 @@
       <c r="M76" s="2" t="s">
         <v>1218</v>
       </c>
-      <c r="N76" s="2">
+      <c r="N76" s="7">
         <v>5</v>
       </c>
       <c r="O76" s="64" t="s">
@@ -10036,7 +10163,7 @@
       <c r="M77" s="2" t="s">
         <v>1218</v>
       </c>
-      <c r="N77" s="2">
+      <c r="N77" s="7">
         <v>9</v>
       </c>
       <c r="O77" s="64" t="s">
@@ -10097,7 +10224,7 @@
       <c r="M78" s="2" t="s">
         <v>1218</v>
       </c>
-      <c r="N78" s="2">
+      <c r="N78" s="7">
         <v>8</v>
       </c>
       <c r="O78" s="64" t="s">
@@ -10158,7 +10285,7 @@
       <c r="M79" s="2" t="s">
         <v>1219</v>
       </c>
-      <c r="N79" s="2">
+      <c r="N79" s="7">
         <v>6</v>
       </c>
       <c r="O79" s="64" t="s">
@@ -10280,7 +10407,7 @@
       <c r="M81" s="2" t="s">
         <v>1219</v>
       </c>
-      <c r="N81" s="2">
+      <c r="N81" s="7">
         <v>7</v>
       </c>
       <c r="O81" s="64" t="s">
@@ -10463,7 +10590,7 @@
       <c r="M84" s="2" t="s">
         <v>1219</v>
       </c>
-      <c r="N84" s="2">
+      <c r="N84" s="7">
         <v>2</v>
       </c>
       <c r="O84" s="64" t="s">
@@ -10646,7 +10773,7 @@
       <c r="M87" s="2" t="s">
         <v>1220</v>
       </c>
-      <c r="N87" s="2">
+      <c r="N87" s="7">
         <v>9</v>
       </c>
       <c r="O87" s="64" t="s">
@@ -10707,7 +10834,7 @@
       <c r="M88" s="2" t="s">
         <v>1220</v>
       </c>
-      <c r="N88" s="2">
+      <c r="N88" s="7">
         <v>8</v>
       </c>
       <c r="O88" s="64" t="s">
@@ -10833,7 +10960,7 @@
       <c r="M90" s="2" t="s">
         <v>1220</v>
       </c>
-      <c r="N90" s="2">
+      <c r="N90" s="7">
         <v>7</v>
       </c>
       <c r="O90" s="64" t="s">
@@ -11215,7 +11342,7 @@
       <c r="M96" s="2" t="s">
         <v>1221</v>
       </c>
-      <c r="N96" s="2">
+      <c r="N96" s="7">
         <v>3</v>
       </c>
       <c r="O96" s="64" t="s">
@@ -11276,7 +11403,7 @@
       <c r="M97" s="2" t="s">
         <v>1221</v>
       </c>
-      <c r="N97" s="2">
+      <c r="N97" s="7">
         <v>5</v>
       </c>
       <c r="O97" s="64" t="s">
@@ -11337,7 +11464,7 @@
       <c r="M98" s="2" t="s">
         <v>1221</v>
       </c>
-      <c r="N98" s="2">
+      <c r="N98" s="7">
         <v>2</v>
       </c>
       <c r="O98" s="64" t="s">
@@ -11398,7 +11525,7 @@
       <c r="M99" s="2" t="s">
         <v>1221</v>
       </c>
-      <c r="N99" s="2">
+      <c r="N99" s="7">
         <v>9</v>
       </c>
       <c r="O99" s="64" t="s">
@@ -11459,7 +11586,7 @@
       <c r="M100" s="2" t="s">
         <v>1221</v>
       </c>
-      <c r="N100" s="2">
+      <c r="N100" s="7">
         <v>1</v>
       </c>
       <c r="O100" s="64" t="s">
@@ -11520,7 +11647,7 @@
       <c r="M101" s="2" t="s">
         <v>1221</v>
       </c>
-      <c r="N101" s="2">
+      <c r="N101" s="7">
         <v>8</v>
       </c>
       <c r="O101" s="64" t="s">
@@ -11581,7 +11708,7 @@
       <c r="M102" s="2" t="s">
         <v>1221</v>
       </c>
-      <c r="N102" s="2">
+      <c r="N102" s="7">
         <v>6</v>
       </c>
       <c r="O102" s="64" t="s">
@@ -11642,7 +11769,7 @@
       <c r="M103" s="2" t="s">
         <v>1221</v>
       </c>
-      <c r="N103" s="2">
+      <c r="N103" s="7">
         <v>7</v>
       </c>
       <c r="O103" s="64" t="s">
@@ -11703,7 +11830,7 @@
       <c r="M104" s="2" t="s">
         <v>1221</v>
       </c>
-      <c r="N104" s="2">
+      <c r="N104" s="7">
         <v>4</v>
       </c>
       <c r="O104" s="64" t="s">
@@ -11759,10 +11886,14 @@
         <v>46197</v>
       </c>
       <c r="L105" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M105" s="2"/>
-      <c r="N105" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M105" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="N105" s="2">
+        <v>9</v>
+      </c>
       <c r="O105" s="64" t="s">
         <v>25</v>
       </c>
@@ -11816,10 +11947,14 @@
         <v>46197</v>
       </c>
       <c r="L106" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M106" s="2"/>
-      <c r="N106" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M106" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="N106" s="2">
+        <v>8</v>
+      </c>
       <c r="O106" s="64" t="s">
         <v>25</v>
       </c>
@@ -11873,10 +12008,14 @@
         <v>46197</v>
       </c>
       <c r="L107" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M107" s="2"/>
-      <c r="N107" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M107" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="N107" s="2">
+        <v>1</v>
+      </c>
       <c r="O107" s="64" t="s">
         <v>132</v>
       </c>
@@ -11930,10 +12069,14 @@
         <v>46197</v>
       </c>
       <c r="L108" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M108" s="2"/>
-      <c r="N108" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M108" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="N108" s="2">
+        <v>7</v>
+      </c>
       <c r="O108" s="64" t="s">
         <v>130</v>
       </c>
@@ -11989,8 +12132,12 @@
       <c r="L109" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M109" s="2"/>
-      <c r="N109" s="2"/>
+      <c r="M109" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="N109" s="7">
+        <v>2</v>
+      </c>
       <c r="O109" s="64" t="s">
         <v>132</v>
       </c>
@@ -12044,10 +12191,14 @@
         <v>46197</v>
       </c>
       <c r="L110" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M110" s="2"/>
-      <c r="N110" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M110" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="N110" s="2">
+        <v>6</v>
+      </c>
       <c r="O110" s="64" t="s">
         <v>130</v>
       </c>
@@ -12101,10 +12252,14 @@
         <v>46197</v>
       </c>
       <c r="L111" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M111" s="2"/>
-      <c r="N111" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M111" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="N111" s="2">
+        <v>3</v>
+      </c>
       <c r="O111" s="64" t="s">
         <v>132</v>
       </c>
@@ -12158,10 +12313,14 @@
         <v>46197</v>
       </c>
       <c r="L112" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M112" s="2"/>
-      <c r="N112" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M112" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="N112" s="2">
+        <v>5</v>
+      </c>
       <c r="O112" s="64" t="s">
         <v>130</v>
       </c>
@@ -12215,10 +12374,14 @@
         <v>46197</v>
       </c>
       <c r="L113" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M113" s="2"/>
-      <c r="N113" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M113" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="N113" s="2">
+        <v>4</v>
+      </c>
       <c r="O113" s="64" t="s">
         <v>132</v>
       </c>
@@ -12797,7 +12960,7 @@
       <c r="M122" s="2" t="s">
         <v>1223</v>
       </c>
-      <c r="N122" s="2">
+      <c r="N122" s="7">
         <v>4</v>
       </c>
       <c r="O122" s="64" t="s">
@@ -12919,7 +13082,7 @@
       <c r="M124" s="2" t="s">
         <v>1223</v>
       </c>
-      <c r="N124" s="2">
+      <c r="N124" s="7">
         <v>3</v>
       </c>
       <c r="O124" s="64" t="s">
@@ -13041,7 +13204,7 @@
       <c r="M126" s="2" t="s">
         <v>1223</v>
       </c>
-      <c r="N126" s="2">
+      <c r="N126" s="7">
         <v>5</v>
       </c>
       <c r="O126" s="64" t="s">
@@ -13102,7 +13265,7 @@
       <c r="M127" s="2" t="s">
         <v>1223</v>
       </c>
-      <c r="N127" s="2">
+      <c r="N127" s="7">
         <v>6</v>
       </c>
       <c r="O127" s="64" t="s">
@@ -13158,10 +13321,14 @@
         <v>46206</v>
       </c>
       <c r="L128" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M128" s="2"/>
-      <c r="N128" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M128" s="2" t="s">
+        <v>1287</v>
+      </c>
+      <c r="N128" s="2">
+        <v>6</v>
+      </c>
       <c r="O128" s="64" t="s">
         <v>25</v>
       </c>
@@ -13215,10 +13382,14 @@
         <v>46206</v>
       </c>
       <c r="L129" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M129" s="2"/>
-      <c r="N129" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M129" s="2" t="s">
+        <v>1287</v>
+      </c>
+      <c r="N129" s="2">
+        <v>4</v>
+      </c>
       <c r="O129" s="64" t="s">
         <v>28</v>
       </c>
@@ -13272,10 +13443,14 @@
         <v>46206</v>
       </c>
       <c r="L130" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M130" s="2"/>
-      <c r="N130" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M130" s="2" t="s">
+        <v>1287</v>
+      </c>
+      <c r="N130" s="2">
+        <v>7</v>
+      </c>
       <c r="O130" s="64" t="s">
         <v>25</v>
       </c>
@@ -13329,10 +13504,14 @@
         <v>46206</v>
       </c>
       <c r="L131" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M131" s="2"/>
-      <c r="N131" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M131" s="2" t="s">
+        <v>1287</v>
+      </c>
+      <c r="N131" s="2">
+        <v>3</v>
+      </c>
       <c r="O131" s="64" t="s">
         <v>28</v>
       </c>
@@ -13386,10 +13565,14 @@
         <v>46206</v>
       </c>
       <c r="L132" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M132" s="2"/>
-      <c r="N132" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M132" s="2" t="s">
+        <v>1287</v>
+      </c>
+      <c r="N132" s="2">
+        <v>5</v>
+      </c>
       <c r="O132" s="64" t="s">
         <v>25</v>
       </c>
@@ -13443,10 +13626,14 @@
         <v>46206</v>
       </c>
       <c r="L133" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M133" s="2"/>
-      <c r="N133" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M133" s="2" t="s">
+        <v>1287</v>
+      </c>
+      <c r="N133" s="2">
+        <v>2</v>
+      </c>
       <c r="O133" s="64" t="s">
         <v>28</v>
       </c>
@@ -13500,10 +13687,14 @@
         <v>46206</v>
       </c>
       <c r="L134" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M134" s="2"/>
-      <c r="N134" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="M134" s="2" t="s">
+        <v>1287</v>
+      </c>
+      <c r="N134" s="2">
+        <v>1</v>
+      </c>
       <c r="O134" s="64" t="s">
         <v>28</v>
       </c>
@@ -13887,7 +14078,7 @@
       <c r="M140" s="2" t="s">
         <v>1225</v>
       </c>
-      <c r="N140" s="2">
+      <c r="N140" s="7">
         <v>5</v>
       </c>
       <c r="O140" s="64" t="s">
@@ -13948,7 +14139,7 @@
       <c r="M141" s="2" t="s">
         <v>1225</v>
       </c>
-      <c r="N141" s="2">
+      <c r="N141" s="7">
         <v>7</v>
       </c>
       <c r="O141" s="64" t="s">
@@ -14009,7 +14200,7 @@
       <c r="M142" s="2" t="s">
         <v>1225</v>
       </c>
-      <c r="N142" s="2">
+      <c r="N142" s="7">
         <v>9</v>
       </c>
       <c r="O142" s="64" t="s">
@@ -14070,7 +14261,7 @@
       <c r="M143" s="2" t="s">
         <v>1225</v>
       </c>
-      <c r="N143" s="2">
+      <c r="N143" s="7">
         <v>3</v>
       </c>
       <c r="O143" s="64" t="s">
@@ -14131,7 +14322,7 @@
       <c r="M144" s="2" t="s">
         <v>1225</v>
       </c>
-      <c r="N144" s="2">
+      <c r="N144" s="7">
         <v>1</v>
       </c>
       <c r="O144" s="64" t="s">
@@ -14192,7 +14383,7 @@
       <c r="M145" s="2" t="s">
         <v>1225</v>
       </c>
-      <c r="N145" s="2">
+      <c r="N145" s="7">
         <v>2</v>
       </c>
       <c r="O145" s="64" t="s">
@@ -14253,7 +14444,7 @@
       <c r="M146" s="2" t="s">
         <v>1225</v>
       </c>
-      <c r="N146" s="2">
+      <c r="N146" s="7">
         <v>8</v>
       </c>
       <c r="O146" s="64" t="s">
@@ -14314,7 +14505,7 @@
       <c r="M147" s="2" t="s">
         <v>1225</v>
       </c>
-      <c r="N147" s="2">
+      <c r="N147" s="7">
         <v>4</v>
       </c>
       <c r="O147" s="64" t="s">
@@ -14375,7 +14566,7 @@
       <c r="M148" s="2" t="s">
         <v>1225</v>
       </c>
-      <c r="N148" s="2">
+      <c r="N148" s="7">
         <v>6</v>
       </c>
       <c r="O148" s="64" t="s">
@@ -14436,7 +14627,7 @@
       <c r="M149" s="2" t="s">
         <v>1226</v>
       </c>
-      <c r="N149" s="2">
+      <c r="N149" s="7">
         <v>1</v>
       </c>
       <c r="O149" s="64" t="s">
@@ -14497,7 +14688,7 @@
       <c r="M150" s="2" t="s">
         <v>1226</v>
       </c>
-      <c r="N150" s="2">
+      <c r="N150" s="7">
         <v>2</v>
       </c>
       <c r="O150" s="64" t="s">
@@ -14558,7 +14749,7 @@
       <c r="M151" s="2" t="s">
         <v>1226</v>
       </c>
-      <c r="N151" s="2">
+      <c r="N151" s="7">
         <v>3</v>
       </c>
       <c r="O151" s="64" t="s">
@@ -14680,7 +14871,7 @@
       <c r="M153" s="2" t="s">
         <v>1226</v>
       </c>
-      <c r="N153" s="2">
+      <c r="N153" s="7">
         <v>5</v>
       </c>
       <c r="O153" s="64" t="s">
@@ -14741,7 +14932,7 @@
       <c r="M154" s="2" t="s">
         <v>1226</v>
       </c>
-      <c r="N154" s="2">
+      <c r="N154" s="7">
         <v>6</v>
       </c>
       <c r="O154" s="64" t="s">
@@ -14863,7 +15054,7 @@
       <c r="M156" s="2" t="s">
         <v>1227</v>
       </c>
-      <c r="N156" s="2">
+      <c r="N156" s="7">
         <v>2</v>
       </c>
       <c r="O156" s="64" t="s">
@@ -14985,7 +15176,7 @@
       <c r="M158" s="2" t="s">
         <v>1227</v>
       </c>
-      <c r="N158" s="2">
+      <c r="N158" s="7">
         <v>4</v>
       </c>
       <c r="O158" s="64" t="s">
@@ -15107,7 +15298,7 @@
       <c r="M160" s="2" t="s">
         <v>1227</v>
       </c>
-      <c r="N160" s="2">
+      <c r="N160" s="7">
         <v>6</v>
       </c>
       <c r="O160" s="64" t="s">
@@ -15360,8 +15551,12 @@
       <c r="L164" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M164" s="2"/>
-      <c r="N164" s="2"/>
+      <c r="M164" s="2" t="s">
+        <v>1284</v>
+      </c>
+      <c r="N164" s="7">
+        <v>1</v>
+      </c>
       <c r="O164" s="64" t="s">
         <v>235</v>
       </c>
@@ -15417,8 +15612,12 @@
       <c r="L165" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M165" s="2"/>
-      <c r="N165" s="2"/>
+      <c r="M165" s="2" t="s">
+        <v>1284</v>
+      </c>
+      <c r="N165" s="7">
+        <v>3</v>
+      </c>
       <c r="O165" s="64" t="s">
         <v>237</v>
       </c>
@@ -15474,8 +15673,12 @@
       <c r="L166" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M166" s="2"/>
-      <c r="N166" s="2"/>
+      <c r="M166" s="2" t="s">
+        <v>1284</v>
+      </c>
+      <c r="N166" s="7">
+        <v>2</v>
+      </c>
       <c r="O166" s="64" t="s">
         <v>235</v>
       </c>
@@ -15531,8 +15734,12 @@
       <c r="L167" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M167" s="2"/>
-      <c r="N167" s="2"/>
+      <c r="M167" s="2" t="s">
+        <v>1284</v>
+      </c>
+      <c r="N167" s="7">
+        <v>4</v>
+      </c>
       <c r="O167" s="64" t="s">
         <v>237</v>
       </c>
@@ -16108,8 +16315,12 @@
       <c r="L176" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M176" s="2"/>
-      <c r="N176" s="2"/>
+      <c r="M176" s="2" t="s">
+        <v>1285</v>
+      </c>
+      <c r="N176" s="7">
+        <v>8</v>
+      </c>
       <c r="O176" s="64" t="s">
         <v>235</v>
       </c>
@@ -16165,8 +16376,12 @@
       <c r="L177" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M177" s="2"/>
-      <c r="N177" s="2"/>
+      <c r="M177" s="2" t="s">
+        <v>1285</v>
+      </c>
+      <c r="N177" s="7">
+        <v>4</v>
+      </c>
       <c r="O177" s="64" t="s">
         <v>237</v>
       </c>
@@ -16222,8 +16437,12 @@
       <c r="L178" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M178" s="2"/>
-      <c r="N178" s="2"/>
+      <c r="M178" s="2" t="s">
+        <v>1285</v>
+      </c>
+      <c r="N178" s="7">
+        <v>7</v>
+      </c>
       <c r="O178" s="64" t="s">
         <v>235</v>
       </c>
@@ -16279,8 +16498,12 @@
       <c r="L179" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M179" s="2"/>
-      <c r="N179" s="2"/>
+      <c r="M179" s="2" t="s">
+        <v>1285</v>
+      </c>
+      <c r="N179" s="7">
+        <v>3</v>
+      </c>
       <c r="O179" s="64" t="s">
         <v>237</v>
       </c>
@@ -16336,8 +16559,12 @@
       <c r="L180" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M180" s="2"/>
-      <c r="N180" s="2"/>
+      <c r="M180" s="2" t="s">
+        <v>1285</v>
+      </c>
+      <c r="N180" s="7">
+        <v>6</v>
+      </c>
       <c r="O180" s="64" t="s">
         <v>235</v>
       </c>
@@ -16393,8 +16620,12 @@
       <c r="L181" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M181" s="2"/>
-      <c r="N181" s="2"/>
+      <c r="M181" s="2" t="s">
+        <v>1285</v>
+      </c>
+      <c r="N181" s="7">
+        <v>1</v>
+      </c>
       <c r="O181" s="64" t="s">
         <v>237</v>
       </c>
@@ -16450,8 +16681,12 @@
       <c r="L182" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M182" s="2"/>
-      <c r="N182" s="2"/>
+      <c r="M182" s="2" t="s">
+        <v>1285</v>
+      </c>
+      <c r="N182" s="7">
+        <v>5</v>
+      </c>
       <c r="O182" s="64" t="s">
         <v>235</v>
       </c>
@@ -16507,8 +16742,12 @@
       <c r="L183" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M183" s="2"/>
-      <c r="N183" s="2"/>
+      <c r="M183" s="2" t="s">
+        <v>1285</v>
+      </c>
+      <c r="N183" s="7">
+        <v>2</v>
+      </c>
       <c r="O183" s="64" t="s">
         <v>28</v>
       </c>
@@ -17080,8 +17319,8 @@
     <col min="11" max="13" width="20.265625" customWidth="1"/>
     <col min="14" max="14" width="35.46484375" customWidth="1"/>
     <col min="15" max="15" width="20.1328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="25.86328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="19.265625" customWidth="1"/>
+    <col min="16" max="16" width="24.59765625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="27.6640625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="22.86328125" customWidth="1"/>
     <col min="19" max="19" width="11.6640625" customWidth="1"/>
   </cols>
@@ -17358,7 +17597,9 @@
       <c r="B6" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="53"/>
+      <c r="C6" s="53" t="s">
+        <v>1281</v>
+      </c>
       <c r="D6" s="53" t="s">
         <v>284</v>
       </c>
@@ -17368,8 +17609,12 @@
       <c r="F6" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
+      <c r="G6" s="3">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="H6" s="57">
+        <v>46255</v>
+      </c>
       <c r="I6" s="21" t="b">
         <v>0</v>
       </c>
@@ -17458,7 +17703,9 @@
       <c r="B8" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="53"/>
+      <c r="C8" s="53" t="s">
+        <v>1282</v>
+      </c>
       <c r="D8" s="53" t="s">
         <v>284</v>
       </c>
@@ -17468,8 +17715,12 @@
       <c r="F8" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="G8" s="3">
+        <v>0.104</v>
+      </c>
+      <c r="H8" s="57">
+        <v>46255</v>
+      </c>
       <c r="I8" s="21" t="b">
         <v>0</v>
       </c>
@@ -25240,7 +25491,9 @@
       <c r="B156" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C156" s="53"/>
+      <c r="C156" s="53" t="s">
+        <v>1280</v>
+      </c>
       <c r="D156" s="53" t="s">
         <v>284</v>
       </c>
@@ -25250,8 +25503,12 @@
       <c r="F156" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G156" s="3"/>
-      <c r="H156" s="3"/>
+      <c r="G156" s="3">
+        <v>7.9000000000000001E-2</v>
+      </c>
+      <c r="H156" s="57">
+        <v>46255</v>
+      </c>
       <c r="I156" s="21" t="b">
         <v>0</v>
       </c>
@@ -25287,7 +25544,9 @@
       <c r="B157" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C157" s="53"/>
+      <c r="C157" s="53" t="s">
+        <v>1279</v>
+      </c>
       <c r="D157" s="53" t="s">
         <v>284</v>
       </c>
@@ -25297,8 +25556,12 @@
       <c r="F157" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G157" s="3"/>
-      <c r="H157" s="3"/>
+      <c r="G157" s="3">
+        <v>8.4000000000000005E-2</v>
+      </c>
+      <c r="H157" s="57">
+        <v>46255</v>
+      </c>
       <c r="I157" s="21" t="b">
         <v>0</v>
       </c>
@@ -25334,7 +25597,9 @@
       <c r="B158" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C158" s="53"/>
+      <c r="C158" s="53" t="s">
+        <v>1278</v>
+      </c>
       <c r="D158" s="53" t="s">
         <v>284</v>
       </c>
@@ -25344,8 +25609,12 @@
       <c r="F158" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G158" s="3"/>
-      <c r="H158" s="3"/>
+      <c r="G158" s="3">
+        <v>0.104</v>
+      </c>
+      <c r="H158" s="57">
+        <v>46255</v>
+      </c>
       <c r="I158" s="21" t="b">
         <v>0</v>
       </c>
@@ -25381,7 +25650,9 @@
       <c r="B159" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C159" s="53"/>
+      <c r="C159" s="53" t="s">
+        <v>1191</v>
+      </c>
       <c r="D159" s="53" t="s">
         <v>284</v>
       </c>
@@ -25391,8 +25662,12 @@
       <c r="F159" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G159" s="3"/>
-      <c r="H159" s="3"/>
+      <c r="G159" s="3" t="s">
+        <v>1191</v>
+      </c>
+      <c r="H159" s="57">
+        <v>46255</v>
+      </c>
       <c r="I159" s="21" t="b">
         <v>0</v>
       </c>
@@ -25428,7 +25703,9 @@
       <c r="B160" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C160" s="53"/>
+      <c r="C160" s="53" t="s">
+        <v>1191</v>
+      </c>
       <c r="D160" s="53" t="s">
         <v>284</v>
       </c>
@@ -25438,8 +25715,12 @@
       <c r="F160" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G160" s="3"/>
-      <c r="H160" s="3"/>
+      <c r="G160" s="3" t="s">
+        <v>1191</v>
+      </c>
+      <c r="H160" s="57">
+        <v>46255</v>
+      </c>
       <c r="I160" s="21" t="b">
         <v>0</v>
       </c>
@@ -25475,7 +25756,9 @@
       <c r="B161" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C161" s="53"/>
+      <c r="C161" s="53" t="s">
+        <v>1191</v>
+      </c>
       <c r="D161" s="53" t="s">
         <v>284</v>
       </c>
@@ -25485,8 +25768,12 @@
       <c r="F161" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="G161" s="3"/>
-      <c r="H161" s="3"/>
+      <c r="G161" s="3" t="s">
+        <v>1191</v>
+      </c>
+      <c r="H161" s="57">
+        <v>46255</v>
+      </c>
       <c r="I161" s="21" t="b">
         <v>0</v>
       </c>

</xml_diff>